<commit_message>
Add strikethrough (~~text~~) support
  - Parse ~~text~~ as strikethrough in StripInlineFormatting and
    ParseRichText, render with Excel Font.Strike in rich text runs
  - Add Strike field to RichTextSegment
  - Add 5 unit tests for strikethrough parsing
  - Update demo.md with strikethrough examples in body text and lists
  - Update README, spec, and unsupported_features.md
</commit_message>
<xml_diff>
--- a/sample/output/demo.xlsx
+++ b/sample/output/demo.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="200">
-  <si>
-    <t>md2xls Feature Demo</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+  <si>
+    <t>1. md2xls Feature Demo</t>
   </si>
   <si>
     <t/>
@@ -28,78 +28,84 @@
     <t>converted to Excel.</t>
   </si>
   <si>
+    <t>1.1. Headings</t>
+  </si>
+  <si>
+    <t>1.1.1. Auto-numbered Headings</t>
+  </si>
+  <si>
+    <t>Headings are automatically numbered based on hierarchy: H1 gets 1., H2 gets 1.1., H3 gets 1.1.1., and H4 gets 1.1.1.1..</t>
+  </si>
+  <si>
+    <t>H5 and H6 are rendered without numbering. This numbering can be disabled via the heading_number: false config option or</t>
+  </si>
+  <si>
+    <t>the --no-heading-number CLI flag.</t>
+  </si>
+  <si>
+    <t>1.1.1.1. H4 Item Heading</t>
+  </si>
+  <si>
+    <t>This is an H4 heading. It should be numbered 1.2.1.1. in the output with 14pt bold font.</t>
+  </si>
+  <si>
+    <t>H5 SubItem Heading</t>
+  </si>
+  <si>
+    <t>This is an H5 heading. It is rendered without numbering, with 12pt bold font.</t>
+  </si>
+  <si>
+    <t>H6 Detail Heading</t>
+  </si>
+  <si>
+    <t>This is an H6 heading. It is rendered without numbering, with 11pt bold italic font.</t>
+  </si>
+  <si>
+    <t>1.1.1.2. Second H4</t>
+  </si>
+  <si>
+    <t>This verifies that the H4 counter increments correctly: 1.2.1.2..</t>
+  </si>
+  <si>
+    <t>1.1.2. Heading Counter Reset</t>
+  </si>
+  <si>
+    <t>After this H3, the H4/H5/H6 counters should reset. The next H4 should be 1.2.2.1..</t>
+  </si>
+  <si>
+    <t>1.1.2.1. Reset Verified</t>
+  </si>
+  <si>
+    <t>This H4 should be 1.2.2.1., not 1.2.2.3..</t>
+  </si>
+  <si>
+    <t>1.2. Tables</t>
+  </si>
+  <si>
+    <t>1.2.1. Basic Table</t>
+  </si>
+  <si>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>Headings</t>
   </si>
   <si>
-    <t>Auto-numbered Headings</t>
-  </si>
-  <si>
-    <t>Headings are automatically numbered based on hierarchy: H1 gets 1., H2 gets 1.1., H3 gets 1.1.1., and H4 gets 1.1.1.1..</t>
-  </si>
-  <si>
-    <t>H5 and H6 are rendered without numbering. This numbering can be disabled via the heading_number: false config option or</t>
-  </si>
-  <si>
-    <t>the --no-heading-number CLI flag.</t>
-  </si>
-  <si>
-    <t>H4 Item Heading</t>
-  </si>
-  <si>
-    <t>This is an H4 heading. It should be numbered 1.2.1.1. in the output with 14pt bold font.</t>
-  </si>
-  <si>
-    <t>H5 SubItem Heading</t>
-  </si>
-  <si>
-    <t>This is an H5 heading. It is rendered without numbering, with 12pt bold font.</t>
-  </si>
-  <si>
-    <t>H6 Detail Heading</t>
-  </si>
-  <si>
-    <t>This is an H6 heading. It is rendered without numbering, with 11pt bold italic font.</t>
-  </si>
-  <si>
-    <t>Second H4</t>
-  </si>
-  <si>
-    <t>This verifies that the H4 counter increments correctly: 1.2.1.2..</t>
-  </si>
-  <si>
-    <t>Heading Counter Reset</t>
-  </si>
-  <si>
-    <t>After this H3, the H4/H5/H6 counters should reset. The next H4 should be 1.2.2.1..</t>
-  </si>
-  <si>
-    <t>Reset Verified</t>
-  </si>
-  <si>
-    <t>This H4 should be 1.2.2.1., not 1.2.2.3..</t>
+    <t>Supported</t>
+  </si>
+  <si>
+    <t>H1-H4 auto-numbered, H5-H6 unnumbered</t>
   </si>
   <si>
     <t>Tables</t>
   </si>
   <si>
-    <t>Basic Table</t>
-  </si>
-  <si>
-    <t>Feature</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Supported</t>
-  </si>
-  <si>
-    <t>H1-H4 auto-numbered, H5-H6 unnumbered</t>
-  </si>
-  <si>
     <t>Header + data rows + alignment</t>
   </si>
   <si>
@@ -133,7 +139,7 @@
     <t>Bold/italic in Excel cells</t>
   </si>
   <si>
-    <t>Table with Column Alignment</t>
+    <t>1.2.2. Table with Column Alignment</t>
   </si>
   <si>
     <t>Left Aligned</t>
@@ -172,7 +178,7 @@
     <t>$3.00</t>
   </si>
   <si>
-    <t>Mixed Alignment Table</t>
+    <t>1.2.3. Mixed Alignment Table</t>
   </si>
   <si>
     <t>ID</t>
@@ -223,7 +229,7 @@
     <t>C+</t>
   </si>
   <si>
-    <t>Wide Column Table</t>
+    <t>1.2.4. Wide Column Table</t>
   </si>
   <si>
     <t>Description</t>
@@ -238,10 +244,10 @@
     <t>Another lengthy cell content designed to test the automatic column merging behavior when data exceeds the eighty byte threshold in md2xls</t>
   </si>
   <si>
-    <t>Code Blocks</t>
-  </si>
-  <si>
-    <t>Go</t>
+    <t>1.3. Code Blocks</t>
+  </si>
+  <si>
+    <t>1.3.1. Go</t>
   </si>
   <si>
     <t>package main
@@ -251,7 +257,7 @@
 }</t>
   </si>
   <si>
-    <t>Python</t>
+    <t>1.3.2. Python</t>
   </si>
   <si>
     <t>def greet(name: str) -&gt; str:
@@ -261,11 +267,14 @@
     print(greet("md2xls"))</t>
   </si>
   <si>
-    <t>No Language Specified</t>
+    <t>1.3.3. No Language Specified</t>
   </si>
   <si>
     <t>This is a plain code block without a language tag.
 It should still render with code styling.</t>
+  </si>
+  <si>
+    <t>1.4. Blockquotes</t>
   </si>
   <si>
     <t>This is a simple blockquote.
@@ -282,13 +291,19 @@
     <t>Bold and italic formatting inside a blockquote is stripped to plain text.</t>
   </si>
   <si>
-    <t>Markdown Image Syntax</t>
-  </si>
-  <si>
-    <t>HTML Image Syntax</t>
-  </si>
-  <si>
-    <t>Unordered List</t>
+    <t>1.5. Images</t>
+  </si>
+  <si>
+    <t>1.5.1. Markdown Image Syntax</t>
+  </si>
+  <si>
+    <t>1.5.2. HTML Image Syntax</t>
+  </si>
+  <si>
+    <t>1.6. Lists</t>
+  </si>
+  <si>
+    <t>1.6.1. Unordered List</t>
   </si>
   <si>
     <t>• First item</t>
@@ -418,7 +433,46 @@
     <t>• Sixth item has inline code in it</t>
   </si>
   <si>
-    <t>Ordered List</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Seventh item with </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <strike val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>strikethrough</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> text</t>
+    </r>
+  </si>
+  <si>
+    <t>1.6.2. Ordered List</t>
   </si>
   <si>
     <t>1. Step one</t>
@@ -430,7 +484,7 @@
     <t>3. Step three</t>
   </si>
   <si>
-    <t>Nested List</t>
+    <t>1.6.3. Nested List</t>
   </si>
   <si>
     <t>• Parent item</t>
@@ -457,7 +511,7 @@
     <t xml:space="preserve">    2. Nested ordered 2</t>
   </si>
   <si>
-    <t>Task Lists</t>
+    <t>1.6.4. Task Lists</t>
   </si>
   <si>
     <t>☐ Design the new feature</t>
@@ -475,7 +529,7 @@
     <t>☐ Write documentation</t>
   </si>
   <si>
-    <t>Nested Task Lists</t>
+    <t>1.6.5. Nested Task Lists</t>
   </si>
   <si>
     <t>☐ Release v2.0</t>
@@ -505,7 +559,7 @@
     <t xml:space="preserve">    ☑ Excel rendering</t>
   </si>
   <si>
-    <t>Mixed Task and Regular Lists</t>
+    <t>1.6.6. Mixed Task and Regular Lists</t>
   </si>
   <si>
     <t>☑ Completed task</t>
@@ -520,7 +574,7 @@
     <t>☑ Another completed task</t>
   </si>
   <si>
-    <t>Links &amp; Hyperlinks</t>
+    <t>1.7. Links &amp; Hyperlinks</t>
   </si>
   <si>
     <t>md2xls on GitHub</t>
@@ -532,7 +586,7 @@
     <t>This line has multiple links inside it.</t>
   </si>
   <si>
-    <t>Links with Rich Text (BUG-M01)</t>
+    <t>1.7.1. Links with Rich Text (BUG-M01)</t>
   </si>
   <si>
     <r>
@@ -625,7 +679,7 @@
     </r>
   </si>
   <si>
-    <t>Inline Formatting (Rich Text)</t>
+    <t>1.8. Inline Formatting (Rich Text)</t>
   </si>
   <si>
     <r>
@@ -723,6 +777,36 @@
       <rPr>
         <rFont val="游ゴシック Regular"/>
         <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This text has </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <strike val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>strikethrough</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> rendered with a line through it.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
         <b val="1"/>
         <color/>
         <sz val="11"/>
@@ -823,6 +907,25 @@
         <color/>
         <sz val="11"/>
       </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <strike val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>strikethrough</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
       <t xml:space="preserve">, and </t>
     </r>
     <r>
@@ -848,7 +951,7 @@
     <t>Plain text without any formatting markers stays as-is.</t>
   </si>
   <si>
-    <t>Inline Code with Asterisks (BUG-H01)</t>
+    <t>1.8.1. Inline Code with Asterisks (BUG-H01)</t>
   </si>
   <si>
     <t>Use *ptr to dereference a pointer in C.</t>
@@ -1009,7 +1112,7 @@
     </r>
   </si>
   <si>
-    <t>HTML Entities</t>
+    <t>1.9. HTML Entities</t>
   </si>
   <si>
     <t>Special characters: &amp; &lt; &gt; "</t>
@@ -1024,7 +1127,7 @@
     <t>Japanese yen sign: ¥ | Registered: ®</t>
   </si>
   <si>
-    <t>Horizontal Rules</t>
+    <t>1.10. Horizontal Rules</t>
   </si>
   <si>
     <t>Above the first rule.</t>
@@ -1039,10 +1142,10 @@
     <t>After the third style of rule.</t>
   </si>
   <si>
-    <t>Text Wrapping</t>
-  </si>
-  <si>
-    <t>Word-Boundary Splitting</t>
+    <t>1.11. Text Wrapping</t>
+  </si>
+  <si>
+    <t>1.11.1. Word-Boundary Splitting</t>
   </si>
   <si>
     <t>The quick brown fox jumps over the lazy dog. This sentence is intentionally long to demonstrate that md2xls now splits</t>
@@ -1054,13 +1157,13 @@
     <t>generated Excel file.</t>
   </si>
   <si>
-    <t>CJK Character Splitting</t>
+    <t>1.11.2. CJK Character Splitting</t>
   </si>
   <si>
     <t>md2xlsは日本語のような文字間にスペースのないテキストについては従来通り文字数ベースで分割します。これにより日本語や中国語などのCJKテキストでも適切に行が折り返されます。</t>
   </si>
   <si>
-    <t>Mixed Content</t>
+    <t>1.11.3. Mixed Content</t>
   </si>
   <si>
     <t>This is a mixed line containing both English and 日本語テキスト together, which tests how the word-boundary-aware splitting</t>
@@ -1069,34 +1172,34 @@
     <t>handles text with a combination of space-separated and non-space-separated characters.</t>
   </si>
   <si>
-    <t>Edge Cases</t>
-  </si>
-  <si>
-    <t>Empty Lines</t>
+    <t>1.12. Edge Cases</t>
+  </si>
+  <si>
+    <t>1.12.1. Empty Lines</t>
   </si>
   <si>
     <t>The lines above and below this text are empty and should render as blank rows.</t>
   </si>
   <si>
-    <t>Heading After Various Elements</t>
-  </si>
-  <si>
-    <t>Second H1</t>
+    <t>1.12.2. Heading After Various Elements</t>
+  </si>
+  <si>
+    <t>2. Second H1</t>
   </si>
   <si>
     <t>This is a second top-level heading, demonstrating that chapter numbering resets sections and terms.</t>
   </si>
   <si>
-    <t>New Section</t>
-  </si>
-  <si>
-    <t>New Subsection</t>
+    <t>2.1. New Section</t>
+  </si>
+  <si>
+    <t>2.1.1. New Subsection</t>
   </si>
   <si>
     <t>This should be numbered 2.1.1. in the output.</t>
   </si>
   <si>
-    <t>Deep Nesting Under Second H1</t>
+    <t>2.1.1.1. Deep Nesting Under Second H1</t>
   </si>
   <si>
     <t>This should be 2.1.1.1. — verifying counters reset properly across H1 boundaries.</t>
@@ -1114,13 +1217,13 @@
     <t>Rendered without numbering (H6 is unnumbered).</t>
   </si>
   <si>
-    <t>Another Subsection</t>
+    <t>2.1.2. Another Subsection</t>
   </si>
   <si>
     <t>And this should be 2.1.2..</t>
   </si>
   <si>
-    <t>Summary</t>
+    <t>2.2. Summary</t>
   </si>
   <si>
     <t>This demo file covers all md2xls features:</t>
@@ -1150,7 +1253,7 @@
     <t>8. Links rendered as Excel hyperlinks (with rich text support)</t>
   </si>
   <si>
-    <t>9. Inline rich text formatting (bold, italic in Excel cells)</t>
+    <t>9. Inline rich text formatting (bold, italic, strikethrough in Excel cells)</t>
   </si>
   <si>
     <t>10. Inline code protection (asterisks inside backticks are not parsed as emphasis)</t>
@@ -1872,79 +1975,79 @@
     </row>
     <row r="43">
       <c r="A43" s="9" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50">
@@ -1954,7 +2057,7 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52">
@@ -1964,46 +2067,46 @@
     </row>
     <row r="53">
       <c r="A53" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="57">
@@ -2013,7 +2116,7 @@
     </row>
     <row r="58">
       <c r="A58" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59">
@@ -2023,58 +2126,58 @@
     </row>
     <row r="60">
       <c r="A60" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="13" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D63" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="64">
@@ -2084,7 +2187,7 @@
     </row>
     <row r="65">
       <c r="A65" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="66">
@@ -2094,37 +2197,37 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C67" s="8"/>
     </row>
     <row r="68" ht="105" customHeight="true">
       <c r="A68" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C68" s="9"/>
     </row>
     <row r="69" ht="105" customHeight="true">
       <c r="A69" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C69" s="9"/>
     </row>
     <row r="70" ht="105" customHeight="true">
       <c r="A70" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C70" s="9"/>
     </row>
@@ -2135,7 +2238,7 @@
     </row>
     <row r="72">
       <c r="A72" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2152,7 +2255,7 @@
     </row>
     <row r="74">
       <c r="A74" s="4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="75">
@@ -2162,7 +2265,7 @@
     </row>
     <row r="76">
       <c r="A76" s="14" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B76" s="14"/>
       <c r="C76" s="14"/>
@@ -2259,7 +2362,7 @@
     </row>
     <row r="86">
       <c r="A86" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87">
@@ -2269,7 +2372,7 @@
     </row>
     <row r="88">
       <c r="A88" s="14" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B88" s="14"/>
       <c r="C88" s="14"/>
@@ -2356,7 +2459,7 @@
     </row>
     <row r="97">
       <c r="A97" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="98">
@@ -2366,7 +2469,7 @@
     </row>
     <row r="99">
       <c r="A99" s="14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B99" s="14"/>
       <c r="C99" s="14"/>
@@ -2413,7 +2516,7 @@
     </row>
     <row r="104">
       <c r="A104" s="3" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -2430,7 +2533,7 @@
     </row>
     <row r="106">
       <c r="A106" s="15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
@@ -2487,7 +2590,7 @@
     </row>
     <row r="112">
       <c r="A112" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="113">
@@ -2497,7 +2600,7 @@
     </row>
     <row r="114">
       <c r="A114" s="15" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
@@ -2534,7 +2637,7 @@
     </row>
     <row r="118">
       <c r="A118" s="15" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -2571,7 +2674,7 @@
     </row>
     <row r="122">
       <c r="A122" s="3" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -2588,7 +2691,7 @@
     </row>
     <row r="124">
       <c r="A124" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="125">
@@ -2603,7 +2706,7 @@
     </row>
     <row r="128">
       <c r="A128" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="129">
@@ -2618,7 +2721,7 @@
     </row>
     <row r="132">
       <c r="A132" s="3" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -2635,7 +2738,7 @@
     </row>
     <row r="134">
       <c r="A134" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="135">
@@ -2645,717 +2748,717 @@
     </row>
     <row r="136">
       <c r="A136" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="s">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="4" t="s">
-        <v>94</v>
+      <c r="A143" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="s">
-        <v>1</v>
+      <c r="A144" s="4" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="s">
-        <v>95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="s">
-        <v>1</v>
+        <v>103</v>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="4" t="s">
-        <v>98</v>
+      <c r="A149" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="s">
-        <v>1</v>
+      <c r="A150" s="4" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="s">
-        <v>99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="s">
-        <v>1</v>
+        <v>112</v>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="4" t="s">
-        <v>107</v>
+      <c r="A160" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="s">
-        <v>1</v>
+      <c r="A161" s="4" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="s">
-        <v>1</v>
+        <v>118</v>
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="4" t="s">
-        <v>113</v>
+      <c r="A168" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="s">
-        <v>1</v>
+      <c r="A169" s="4" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="s">
-        <v>114</v>
+        <v>1</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="4" t="s">
-        <v>123</v>
+      <c r="A180" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="s">
-        <v>1</v>
+      <c r="A181" s="4" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="s">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B187" s="3"/>
-      <c r="C187" s="3"/>
-      <c r="D187" s="3"/>
-      <c r="E187" s="3"/>
-      <c r="F187" s="3"/>
-      <c r="G187" s="3"/>
-      <c r="H187" s="3"/>
+      <c r="A187" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A188" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B188" s="3"/>
+      <c r="C188" s="3"/>
+      <c r="D188" s="3"/>
+      <c r="E188" s="3"/>
+      <c r="F188" s="3"/>
+      <c r="G188" s="3"/>
+      <c r="H188" s="3"/>
     </row>
     <row r="189">
-      <c r="A189" s="16" t="s">
-        <v>129</v>
+      <c r="A189" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="s">
-        <v>1</v>
+      <c r="A190" s="16" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="16" t="s">
-        <v>130</v>
+      <c r="A191" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="s">
-        <v>1</v>
+      <c r="A192" s="16" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="16" t="s">
-        <v>131</v>
+      <c r="A193" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="s">
-        <v>1</v>
+      <c r="A194" s="16" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="4" t="s">
-        <v>132</v>
+      <c r="A195" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="s">
-        <v>1</v>
+      <c r="A196" s="4" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="s">
-        <v>133</v>
+        <v>1</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="s">
-        <v>1</v>
+        <v>139</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="s">
-        <v>134</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="s">
-        <v>1</v>
+        <v>140</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="s">
-        <v>135</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="s">
-        <v>1</v>
+        <v>141</v>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B203" s="3"/>
-      <c r="C203" s="3"/>
-      <c r="D203" s="3"/>
-      <c r="E203" s="3"/>
-      <c r="F203" s="3"/>
-      <c r="G203" s="3"/>
-      <c r="H203" s="3"/>
+      <c r="A203" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A204" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B204" s="3"/>
+      <c r="C204" s="3"/>
+      <c r="D204" s="3"/>
+      <c r="E204" s="3"/>
+      <c r="F204" s="3"/>
+      <c r="G204" s="3"/>
+      <c r="H204" s="3"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="s">
-        <v>137</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="s">
-        <v>1</v>
+        <v>143</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="s">
-        <v>138</v>
+        <v>1</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="s">
-        <v>1</v>
+        <v>144</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="s">
-        <v>139</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="s">
-        <v>1</v>
+        <v>145</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="s">
-        <v>140</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="s">
-        <v>1</v>
+        <v>146</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="s">
-        <v>141</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="s">
-        <v>1</v>
+        <v>147</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="s">
-        <v>142</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="s">
-        <v>1</v>
+        <v>148</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="4" t="s">
-        <v>143</v>
+      <c r="A217" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="s">
-        <v>1</v>
+        <v>149</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="s">
-        <v>144</v>
+        <v>1</v>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="s">
-        <v>1</v>
+      <c r="A220" s="4" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="s">
-        <v>145</v>
+        <v>1</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="s">
-        <v>146</v>
+        <v>1</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="s">
-        <v>1</v>
+        <v>152</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="s">
-        <v>147</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B227" s="3"/>
-      <c r="C227" s="3"/>
-      <c r="D227" s="3"/>
-      <c r="E227" s="3"/>
-      <c r="F227" s="3"/>
-      <c r="G227" s="3"/>
-      <c r="H227" s="3"/>
+      <c r="A227" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="s">
-        <v>1</v>
+        <v>154</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="s">
-        <v>149</v>
+        <v>1</v>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A230" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B230" s="3"/>
+      <c r="C230" s="3"/>
+      <c r="D230" s="3"/>
+      <c r="E230" s="3"/>
+      <c r="F230" s="3"/>
+      <c r="G230" s="3"/>
+      <c r="H230" s="3"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="s">
-        <v>150</v>
+        <v>1</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="s">
-        <v>1</v>
+        <v>156</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="s">
-        <v>151</v>
+        <v>1</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="s">
-        <v>1</v>
+        <v>157</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="s">
-        <v>152</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="s">
-        <v>1</v>
+        <v>158</v>
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B237" s="3"/>
-      <c r="C237" s="3"/>
-      <c r="D237" s="3"/>
-      <c r="E237" s="3"/>
-      <c r="F237" s="3"/>
-      <c r="G237" s="3"/>
-      <c r="H237" s="3"/>
+      <c r="A237" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="s">
-        <v>1</v>
+        <v>159</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="s">
-        <v>154</v>
+        <v>1</v>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="241" ht="8" customHeight="true">
-      <c r="A241" s="17"/>
-      <c r="B241" s="17"/>
-      <c r="C241" s="17"/>
-      <c r="D241" s="17"/>
-      <c r="E241" s="17"/>
-      <c r="F241" s="17"/>
-      <c r="G241" s="17"/>
-      <c r="H241" s="17"/>
+      <c r="A240" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B240" s="3"/>
+      <c r="C240" s="3"/>
+      <c r="D240" s="3"/>
+      <c r="E240" s="3"/>
+      <c r="F240" s="3"/>
+      <c r="G240" s="3"/>
+      <c r="H240" s="3"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="s">
-        <v>1</v>
+        <v>161</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="245" ht="8" customHeight="true">
-      <c r="A245" s="17"/>
-      <c r="B245" s="17"/>
-      <c r="C245" s="17"/>
-      <c r="D245" s="17"/>
-      <c r="E245" s="17"/>
-      <c r="F245" s="17"/>
-      <c r="G245" s="17"/>
-      <c r="H245" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" ht="8" customHeight="true">
+      <c r="A244" s="17"/>
+      <c r="B244" s="17"/>
+      <c r="C244" s="17"/>
+      <c r="D244" s="17"/>
+      <c r="E244" s="17"/>
+      <c r="F244" s="17"/>
+      <c r="G244" s="17"/>
+      <c r="H244" s="17"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="s">
-        <v>1</v>
+        <v>162</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="249" ht="8" customHeight="true">
-      <c r="A249" s="17"/>
-      <c r="B249" s="17"/>
-      <c r="C249" s="17"/>
-      <c r="D249" s="17"/>
-      <c r="E249" s="17"/>
-      <c r="F249" s="17"/>
-      <c r="G249" s="17"/>
-      <c r="H249" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" ht="8" customHeight="true">
+      <c r="A248" s="17"/>
+      <c r="B248" s="17"/>
+      <c r="C248" s="17"/>
+      <c r="D248" s="17"/>
+      <c r="E248" s="17"/>
+      <c r="F248" s="17"/>
+      <c r="G248" s="17"/>
+      <c r="H248" s="17"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="s">
-        <v>1</v>
+        <v>163</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="2" t="s">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252" ht="8" customHeight="true">
+      <c r="A252" s="17"/>
+      <c r="B252" s="17"/>
+      <c r="C252" s="17"/>
+      <c r="D252" s="17"/>
+      <c r="E252" s="17"/>
+      <c r="F252" s="17"/>
+      <c r="G252" s="17"/>
+      <c r="H252" s="17"/>
     </row>
     <row r="253">
-      <c r="A253" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B253" s="3"/>
-      <c r="C253" s="3"/>
-      <c r="D253" s="3"/>
-      <c r="E253" s="3"/>
-      <c r="F253" s="3"/>
-      <c r="G253" s="3"/>
-      <c r="H253" s="3"/>
+      <c r="A253" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="s">
-        <v>1</v>
+        <v>164</v>
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="4" t="s">
-        <v>159</v>
+      <c r="A255" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A256" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B256" s="3"/>
+      <c r="C256" s="3"/>
+      <c r="D256" s="3"/>
+      <c r="E256" s="3"/>
+      <c r="F256" s="3"/>
+      <c r="G256" s="3"/>
+      <c r="H256" s="3"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="s">
-        <v>160</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="s">
-        <v>161</v>
+      <c r="A258" s="4" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="s">
-        <v>162</v>
+        <v>1</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="s">
-        <v>1</v>
+        <v>167</v>
       </c>
     </row>
     <row r="261">
-      <c r="A261" s="4" t="s">
-        <v>163</v>
+      <c r="A261" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="s">
-        <v>1</v>
+        <v>169</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="s">
-        <v>164</v>
+        <v>1</v>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="s">
-        <v>1</v>
+      <c r="A264" s="4" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="4" t="s">
-        <v>165</v>
+      <c r="A265" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="s">
-        <v>1</v>
+        <v>171</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="s">
-        <v>166</v>
+        <v>1</v>
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="s">
-        <v>167</v>
+      <c r="A268" s="4" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="269">
@@ -3364,283 +3467,298 @@
       </c>
     </row>
     <row r="270">
-      <c r="A270" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B270" s="3"/>
-      <c r="C270" s="3"/>
-      <c r="D270" s="3"/>
-      <c r="E270" s="3"/>
-      <c r="F270" s="3"/>
-      <c r="G270" s="3"/>
-      <c r="H270" s="3"/>
+      <c r="A270" s="2" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="s">
-        <v>1</v>
+        <v>174</v>
       </c>
     </row>
     <row r="272">
-      <c r="A272" s="4" t="s">
-        <v>169</v>
+      <c r="A272" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A273" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B273" s="3"/>
+      <c r="C273" s="3"/>
+      <c r="D273" s="3"/>
+      <c r="E273" s="3"/>
+      <c r="F273" s="3"/>
+      <c r="G273" s="3"/>
+      <c r="H273" s="3"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="s">
-        <v>170</v>
+        <v>1</v>
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="s">
-        <v>1</v>
+      <c r="A275" s="4" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="276">
-      <c r="A276" s="4" t="s">
-        <v>171</v>
+      <c r="A276" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="s">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="1" t="s">
-        <v>172</v>
+      <c r="A278" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="s">
-        <v>1</v>
+      <c r="A279" s="4" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="s">
-        <v>173</v>
+        <v>1</v>
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="s">
-        <v>1</v>
+      <c r="A281" s="1" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="282">
-      <c r="A282" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B282" s="3"/>
-      <c r="C282" s="3"/>
-      <c r="D282" s="3"/>
-      <c r="E282" s="3"/>
-      <c r="F282" s="3"/>
-      <c r="G282" s="3"/>
-      <c r="H282" s="3"/>
+      <c r="A282" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="s">
-        <v>1</v>
+        <v>180</v>
       </c>
     </row>
     <row r="284">
-      <c r="A284" s="4" t="s">
-        <v>175</v>
+      <c r="A284" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A285" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B285" s="3"/>
+      <c r="C285" s="3"/>
+      <c r="D285" s="3"/>
+      <c r="E285" s="3"/>
+      <c r="F285" s="3"/>
+      <c r="G285" s="3"/>
+      <c r="H285" s="3"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="s">
-        <v>176</v>
+        <v>1</v>
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="2" t="s">
-        <v>1</v>
+      <c r="A287" s="4" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="5" t="s">
-        <v>177</v>
+      <c r="A288" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="s">
-        <v>1</v>
+        <v>183</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="s">
-        <v>178</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="s">
-        <v>1</v>
+      <c r="A291" s="5" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="6" t="s">
-        <v>179</v>
+      <c r="A292" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="s">
-        <v>1</v>
+        <v>185</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="s">
-        <v>180</v>
+        <v>1</v>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="s">
-        <v>1</v>
+      <c r="A295" s="6" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="7" t="s">
-        <v>181</v>
+      <c r="A296" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="s">
-        <v>1</v>
+        <v>187</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="s">
-        <v>182</v>
+        <v>1</v>
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="2" t="s">
-        <v>1</v>
+      <c r="A299" s="7" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="4" t="s">
-        <v>183</v>
+      <c r="A300" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="s">
-        <v>1</v>
+        <v>189</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="s">
-        <v>184</v>
+        <v>1</v>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="s">
-        <v>1</v>
+      <c r="A303" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="B304" s="3"/>
-      <c r="C304" s="3"/>
-      <c r="D304" s="3"/>
-      <c r="E304" s="3"/>
-      <c r="F304" s="3"/>
-      <c r="G304" s="3"/>
-      <c r="H304" s="3"/>
+      <c r="A304" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="s">
-        <v>1</v>
+        <v>191</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="s">
-        <v>186</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A307" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B307" s="3"/>
+      <c r="C307" s="3"/>
+      <c r="D307" s="3"/>
+      <c r="E307" s="3"/>
+      <c r="F307" s="3"/>
+      <c r="G307" s="3"/>
+      <c r="H307" s="3"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="s">
-        <v>187</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="s">
-        <v>189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3658,12 +3776,12 @@
     <mergeCell ref="A118:H120"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A189" r:id="rId1"/>
-    <hyperlink ref="A191" r:id="rId2"/>
-    <hyperlink ref="A193" r:id="rId3"/>
-    <hyperlink ref="A197" r:id="rId4"/>
-    <hyperlink ref="A199" r:id="rId5"/>
-    <hyperlink ref="A201" r:id="rId6"/>
+    <hyperlink ref="A190" r:id="rId1"/>
+    <hyperlink ref="A192" r:id="rId2"/>
+    <hyperlink ref="A194" r:id="rId3"/>
+    <hyperlink ref="A198" r:id="rId4"/>
+    <hyperlink ref="A200" r:id="rId5"/>
+    <hyperlink ref="A202" r:id="rId6"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add multiple parser and renderer features
  - Add underscore emphasis (__bold__, _italic_) with word-boundary
    protection for snake_case
  - Add inline code font rendering using configured code.font
  - Add rich text preservation across line splits (SplitRichTextPer)
  - Add autolink support (<https://...\>\) with source-order preservation
  - Add HTML comment removal (single-line, multi-line, and inline)
  - Add link/image title attribute stripping ([text](url title))
  - Add configurable heading font sizes (heading_font_size.h1-h6)
  - Add configurable sheet name (sheet_name)
  - Fix tmp/ cleanup to use os.MkdirTemp instead of deleting ./tmp
  - Update README, demo.md, and .m2x.yml with new features
</commit_message>
<xml_diff>
--- a/sample/output/demo.xlsx
+++ b/sample/output/demo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
   <si>
     <t>1. md2xls Feature Demo</t>
   </si>
@@ -34,19 +34,177 @@
     <t>1.1.1. Auto-numbered Headings</t>
   </si>
   <si>
-    <t>Headings are automatically numbered based on hierarchy: H1 gets 1., H2 gets 1.1., H3 gets 1.1.1., and H4 gets 1.1.1.1..</t>
-  </si>
-  <si>
-    <t>H5 and H6 are rendered without numbering. This numbering can be disabled via the heading_number: false config option or</t>
-  </si>
-  <si>
-    <t>the --no-heading-number CLI flag.</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Headings are automatically numbered based on hierarchy: H1 gets </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">, H2 gets </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">, H3 gets </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">, and H4 gets </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.1.1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">H5 and H6 are rendered without numbering. This numbering can be disabled via the </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>heading_number: false</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> config option or</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">the </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>--no-heading-number</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> CLI flag.</t>
+    </r>
   </si>
   <si>
     <t>1.1.1.1. H4 Item Heading</t>
   </si>
   <si>
-    <t>This is an H4 heading. It should be numbered 1.2.1.1. in the output with 14pt bold font.</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This is an H4 heading. It should be numbered </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.2.1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> in the output with 14pt bold font.</t>
+    </r>
   </si>
   <si>
     <t>H5 SubItem Heading</t>
@@ -64,19 +222,115 @@
     <t>1.1.1.2. Second H4</t>
   </si>
   <si>
-    <t>This verifies that the H4 counter increments correctly: 1.2.1.2..</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This verifies that the H4 counter increments correctly: </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.2.1.2.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
   <si>
     <t>1.1.2. Heading Counter Reset</t>
   </si>
   <si>
-    <t>After this H3, the H4/H5/H6 counters should reset. The next H4 should be 1.2.2.1..</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">After this H3, the H4/H5/H6 counters should reset. The next H4 should be </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.2.2.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
   <si>
     <t>1.1.2.1. Reset Verified</t>
   </si>
   <si>
-    <t>This H4 should be 1.2.2.1., not 1.2.2.3..</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This H4 should be </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.2.2.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">, not </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>1.2.2.3.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
   <si>
     <t>1.2. Tables</t>
@@ -300,6 +554,9 @@
     <t>1.5.2. HTML Image Syntax</t>
   </si>
   <si>
+    <t>1.5.3. Image with Title Attribute</t>
+  </si>
+  <si>
     <t>1.6. Lists</t>
   </si>
   <si>
@@ -430,9 +687,6 @@
     </r>
   </si>
   <si>
-    <t>• Sixth item has inline code in it</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="游ゴシック Regular"/>
@@ -449,6 +703,44 @@
         <color/>
         <sz val="11"/>
       </rPr>
+      <t xml:space="preserve">Sixth item has </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>inline code</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> in it (rendered with code font)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
       <t xml:space="preserve">Seventh item with </t>
     </r>
     <r>
@@ -460,6 +752,84 @@
         <sz val="11"/>
       </rPr>
       <t>strikethrough</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> text</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Eighth item with </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> text</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Ninth item with </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore italic</t>
     </r>
     <r>
       <rPr>
@@ -679,7 +1049,31 @@
     </r>
   </si>
   <si>
-    <t>1.8. Inline Formatting (Rich Text)</t>
+    <t>1.7.2. Links with Title Attribute</t>
+  </si>
+  <si>
+    <t>Link with title should show URL without the title text.</t>
+  </si>
+  <si>
+    <t>1.7.3. Autolinks</t>
+  </si>
+  <si>
+    <t>Visit https://go.dev for the official Go site.</t>
+  </si>
+  <si>
+    <t>Both http://example.com and https://example.com are recognized.</t>
+  </si>
+  <si>
+    <t>This line mixes a regular link with https://example.com/b an autolink.</t>
+  </si>
+  <si>
+    <t>1.8. HTML Comments</t>
+  </si>
+  <si>
+    <t>This text is visible.  And this text is also visible.</t>
+  </si>
+  <si>
+    <t>1.9. Inline Formatting (Rich Text)</t>
   </si>
   <si>
     <r>
@@ -930,10 +1324,10 @@
     </r>
     <r>
       <rPr>
-        <rFont val="游ゴシック Regular"/>
-        <family val="2"/>
-        <color/>
-        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
       </rPr>
       <t>inline code</t>
     </r>
@@ -948,16 +1342,425 @@
     </r>
   </si>
   <si>
+    <t>1.9.1. Underscore Emphasis</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This text has </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> rendered the same as </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>asterisk bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This text has </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore italic</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> rendered the same as </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>asterisk italic</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This text has </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore bold italic</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> rendered the same as </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>asterisk bold italic</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>The word snake_case_name should NOT be treated as italic — word boundaries are respected.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Mixed: </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>asterisk bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>underscore bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> in the same line.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.9.2. Inline Code with Code Font</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>inline code</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> in this line should render with the configured code font (e.g., Arial).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Mix of </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>bold text</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>code text</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> shows both formatting and code font in one cell.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.9.3. Rich Text in Long Lines</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This is a very long line with </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>bold formatting</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> that should exceed the max_num_of_characters_per_line limit and</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>demonstrate that bold/italic/strikethrough formatting is preserved even when the text is split across multiple Excel</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>rows, unlike the previous behavior where it fell back to plain text.</t>
+    </r>
+  </si>
+  <si>
     <t>Plain text without any formatting markers stays as-is.</t>
   </si>
   <si>
-    <t>1.8.1. Inline Code with Asterisks (BUG-H01)</t>
-  </si>
-  <si>
-    <t>Use *ptr to dereference a pointer in C.</t>
-  </si>
-  <si>
-    <t>The flags *kwargs and args are Python conventions.</t>
+    <t>1.9.4. Inline Code with Asterisks (BUG-H01)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Use </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>*ptr</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> to dereference a pointer in C.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">The flags </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>**kwargs</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>*args</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> are Python conventions.</t>
+    </r>
   </si>
   <si>
     <r>
@@ -990,10 +1793,10 @@
     </r>
     <r>
       <rPr>
-        <rFont val="游ゴシック Regular"/>
-        <family val="2"/>
-        <color/>
-        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
       </rPr>
       <t>*literal asterisk*</t>
     </r>
@@ -1057,10 +1860,10 @@
     </r>
     <r>
       <rPr>
-        <rFont val="游ゴシック Regular"/>
-        <family val="2"/>
-        <color/>
-        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
       </rPr>
       <t>**not bold**</t>
     </r>
@@ -1094,10 +1897,10 @@
     </r>
     <r>
       <rPr>
-        <rFont val="游ゴシック Regular"/>
-        <family val="2"/>
-        <color/>
-        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
       </rPr>
       <t>*not italic*</t>
     </r>
@@ -1112,7 +1915,7 @@
     </r>
   </si>
   <si>
-    <t>1.9. HTML Entities</t>
+    <t>1.10. HTML Entities</t>
   </si>
   <si>
     <t>Special characters: &amp; &lt; &gt; "</t>
@@ -1127,7 +1930,7 @@
     <t>Japanese yen sign: ¥ | Registered: ®</t>
   </si>
   <si>
-    <t>1.10. Horizontal Rules</t>
+    <t>1.11. Horizontal Rules</t>
   </si>
   <si>
     <t>Above the first rule.</t>
@@ -1142,10 +1945,10 @@
     <t>After the third style of rule.</t>
   </si>
   <si>
-    <t>1.11. Text Wrapping</t>
-  </si>
-  <si>
-    <t>1.11.1. Word-Boundary Splitting</t>
+    <t>1.12. Text Wrapping</t>
+  </si>
+  <si>
+    <t>1.12.1. Word-Boundary Splitting</t>
   </si>
   <si>
     <t>The quick brown fox jumps over the lazy dog. This sentence is intentionally long to demonstrate that md2xls now splits</t>
@@ -1157,13 +1960,13 @@
     <t>generated Excel file.</t>
   </si>
   <si>
-    <t>1.11.2. CJK Character Splitting</t>
+    <t>1.12.2. CJK Character Splitting</t>
   </si>
   <si>
     <t>md2xlsは日本語のような文字間にスペースのないテキストについては従来通り文字数ベースで分割します。これにより日本語や中国語などのCJKテキストでも適切に行が折り返されます。</t>
   </si>
   <si>
-    <t>1.11.3. Mixed Content</t>
+    <t>1.12.3. Mixed Content</t>
   </si>
   <si>
     <t>This is a mixed line containing both English and 日本語テキスト together, which tests how the word-boundary-aware splitting</t>
@@ -1172,16 +1975,16 @@
     <t>handles text with a combination of space-separated and non-space-separated characters.</t>
   </si>
   <si>
-    <t>1.12. Edge Cases</t>
-  </si>
-  <si>
-    <t>1.12.1. Empty Lines</t>
+    <t>1.13. Edge Cases</t>
+  </si>
+  <si>
+    <t>1.13.1. Empty Lines</t>
   </si>
   <si>
     <t>The lines above and below this text are empty and should render as blank rows.</t>
   </si>
   <si>
-    <t>1.12.2. Heading After Various Elements</t>
+    <t>1.13.2. Heading After Various Elements</t>
   </si>
   <si>
     <t>2. Second H1</t>
@@ -1196,13 +1999,65 @@
     <t>2.1.1. New Subsection</t>
   </si>
   <si>
-    <t>This should be numbered 2.1.1. in the output.</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This should be numbered </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>2.1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> in the output.</t>
+    </r>
   </si>
   <si>
     <t>2.1.1.1. Deep Nesting Under Second H1</t>
   </si>
   <si>
-    <t>This should be 2.1.1.1. — verifying counters reset properly across H1 boundaries.</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">This should be </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>2.1.1.1.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> — verifying counters reset properly across H1 boundaries.</t>
+    </r>
   </si>
   <si>
     <t>Even Deeper</t>
@@ -1220,7 +2075,33 @@
     <t>2.1.2. Another Subsection</t>
   </si>
   <si>
-    <t>And this should be 2.1.2..</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">And this should be </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>2.1.2.</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
   <si>
     <t>2.2. Summary</t>
@@ -1241,7 +2122,7 @@
     <t>4. Blockquotes with styling</t>
   </si>
   <si>
-    <t>5. Images (Markdown and HTML syntax)</t>
+    <t>5. Images (Markdown and HTML syntax, title attribute stripped)</t>
   </si>
   <si>
     <t>6. Lists (ordered, unordered, nested) with rich text formatting</t>
@@ -1250,22 +2131,98 @@
     <t>7. Task lists with checkboxes</t>
   </si>
   <si>
-    <t>8. Links rendered as Excel hyperlinks (with rich text support)</t>
-  </si>
-  <si>
-    <t>9. Inline rich text formatting (bold, italic, strikethrough in Excel cells)</t>
-  </si>
-  <si>
-    <t>10. Inline code protection (asterisks inside backticks are not parsed as emphasis)</t>
-  </si>
-  <si>
-    <t>11. HTML entity decoding</t>
-  </si>
-  <si>
-    <t>12. Horizontal rules</t>
-  </si>
-  <si>
-    <t>13. Word-boundary-aware text wrapping</t>
+    <t>8. Links rendered as Excel hyperlinks (title attribute stripped, rich text support)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">9. </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>Autolinks (</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>https://...</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>) rendered as Excel hyperlinks</t>
+    </r>
+  </si>
+  <si>
+    <t>10. Inline rich text formatting (bold, italic, strikethrough — asterisk and underscore syntax)</t>
+  </si>
+  <si>
+    <t>11. Inline code rendered with code font in rich text mode</t>
+  </si>
+  <si>
+    <t>12. Rich text formatting preserved across line splits</t>
+  </si>
+  <si>
+    <t>13. Inline code protection (asterisks inside backticks are not parsed as emphasis)</t>
+  </si>
+  <si>
+    <t>14. HTML comment removal (full-line and inline)</t>
+  </si>
+  <si>
+    <t>15. HTML entity decoding</t>
+  </si>
+  <si>
+    <t>16. Horizontal rules</t>
+  </si>
+  <si>
+    <t>17. Word-boundary-aware text wrapping</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">18. </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Configurable heading font sizes and sheet name via </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>.m2x.yml</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2720,95 +3677,90 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="3" t="s">
+      <c r="A132" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B132" s="3"/>
-      <c r="C132" s="3"/>
-      <c r="D132" s="3"/>
-      <c r="E132" s="3"/>
-      <c r="F132" s="3"/>
-      <c r="G132" s="3"/>
-      <c r="H132" s="3"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
     <row r="135">
       <c r="A135" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="s">
-        <v>93</v>
-      </c>
+      <c r="A136" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B136" s="3"/>
+      <c r="C136" s="3"/>
+      <c r="D136" s="3"/>
+      <c r="E136" s="3"/>
+      <c r="F136" s="3"/>
+      <c r="G136" s="3"/>
+      <c r="H136" s="3"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="s">
-        <v>95</v>
+      <c r="A138" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="s">
-        <v>96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="s">
-        <v>1</v>
+        <v>97</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="4" t="s">
-        <v>100</v>
+      <c r="A144" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="s">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="149">
@@ -2818,7 +3770,7 @@
     </row>
     <row r="150">
       <c r="A150" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="151">
@@ -2828,82 +3780,82 @@
     </row>
     <row r="152">
       <c r="A152" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="s">
-        <v>109</v>
+      <c r="A156" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="s">
-        <v>110</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="s">
-        <v>1</v>
+        <v>110</v>
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="4" t="s">
-        <v>113</v>
+      <c r="A161" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="s">
-        <v>1</v>
+        <v>112</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="s">
-        <v>117</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="s">
-        <v>118</v>
+      <c r="A167" s="4" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="168">
@@ -2912,129 +3864,122 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="4" t="s">
-        <v>119</v>
+      <c r="A169" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="s">
-        <v>1</v>
+        <v>118</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="s">
-        <v>123</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="s">
-        <v>124</v>
+      <c r="A175" s="4" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="s">
-        <v>125</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="s">
-        <v>1</v>
+        <v>126</v>
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="4" t="s">
-        <v>129</v>
+      <c r="A181" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="s">
-        <v>133</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="s">
-        <v>1</v>
+      <c r="A187" s="4" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B188" s="3"/>
-      <c r="C188" s="3"/>
-      <c r="D188" s="3"/>
-      <c r="E188" s="3"/>
-      <c r="F188" s="3"/>
-      <c r="G188" s="3"/>
-      <c r="H188" s="3"/>
+      <c r="A188" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="s">
-        <v>1</v>
+        <v>133</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="16" t="s">
-        <v>135</v>
+      <c r="A190" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="s">
-        <v>1</v>
+        <v>135</v>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="16" t="s">
+      <c r="A192" s="2" t="s">
         <v>136</v>
       </c>
     </row>
@@ -3044,9 +3989,16 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="16" t="s">
+      <c r="A194" s="3" t="s">
         <v>137</v>
       </c>
+      <c r="B194" s="3"/>
+      <c r="C194" s="3"/>
+      <c r="D194" s="3"/>
+      <c r="E194" s="3"/>
+      <c r="F194" s="3"/>
+      <c r="G194" s="3"/>
+      <c r="H194" s="3"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="s">
@@ -3054,7 +4006,7 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="4" t="s">
+      <c r="A196" s="16" t="s">
         <v>138</v>
       </c>
     </row>
@@ -3064,7 +4016,7 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="s">
+      <c r="A198" s="16" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3074,7 +4026,7 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="s">
+      <c r="A200" s="16" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3084,7 +4036,7 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="s">
+      <c r="A202" s="4" t="s">
         <v>141</v>
       </c>
     </row>
@@ -3094,16 +4046,9 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="3" t="s">
+      <c r="A204" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B204" s="3"/>
-      <c r="C204" s="3"/>
-      <c r="D204" s="3"/>
-      <c r="E204" s="3"/>
-      <c r="F204" s="3"/>
-      <c r="G204" s="3"/>
-      <c r="H204" s="3"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="s">
@@ -3131,7 +4076,7 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="s">
+      <c r="A210" s="4" t="s">
         <v>145</v>
       </c>
     </row>
@@ -3141,7 +4086,7 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="s">
+      <c r="A212" s="16" t="s">
         <v>146</v>
       </c>
     </row>
@@ -3151,7 +4096,7 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="s">
+      <c r="A214" s="4" t="s">
         <v>147</v>
       </c>
     </row>
@@ -3161,7 +4106,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="s">
+      <c r="A216" s="16" t="s">
         <v>148</v>
       </c>
     </row>
@@ -3171,7 +4116,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="s">
+      <c r="A218" s="16" t="s">
         <v>149</v>
       </c>
     </row>
@@ -3181,7 +4126,7 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="4" t="s">
+      <c r="A220" s="16" t="s">
         <v>150</v>
       </c>
     </row>
@@ -3191,9 +4136,16 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="s">
+      <c r="A222" s="3" t="s">
         <v>151</v>
       </c>
+      <c r="B222" s="3"/>
+      <c r="C222" s="3"/>
+      <c r="D222" s="3"/>
+      <c r="E222" s="3"/>
+      <c r="F222" s="3"/>
+      <c r="G222" s="3"/>
+      <c r="H222" s="3"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="s">
@@ -3202,17 +4154,17 @@
     </row>
     <row r="224">
       <c r="A224" s="2" t="s">
-        <v>152</v>
+        <v>1</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="s">
-        <v>1</v>
+        <v>152</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="s">
-        <v>153</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227">
@@ -3221,9 +4173,16 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="s">
-        <v>154</v>
-      </c>
+      <c r="A228" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B228" s="3"/>
+      <c r="C228" s="3"/>
+      <c r="D228" s="3"/>
+      <c r="E228" s="3"/>
+      <c r="F228" s="3"/>
+      <c r="G228" s="3"/>
+      <c r="H228" s="3"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="s">
@@ -3231,16 +4190,9 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B230" s="3"/>
-      <c r="C230" s="3"/>
-      <c r="D230" s="3"/>
-      <c r="E230" s="3"/>
-      <c r="F230" s="3"/>
-      <c r="G230" s="3"/>
-      <c r="H230" s="3"/>
+      <c r="A230" s="2" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="s">
@@ -3249,7 +4201,7 @@
     </row>
     <row r="232">
       <c r="A232" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="233">
@@ -3259,7 +4211,7 @@
     </row>
     <row r="234">
       <c r="A234" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="235">
@@ -3269,7 +4221,7 @@
     </row>
     <row r="236">
       <c r="A236" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="237">
@@ -3279,7 +4231,7 @@
     </row>
     <row r="238">
       <c r="A238" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="239">
@@ -3288,16 +4240,9 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="B240" s="3"/>
-      <c r="C240" s="3"/>
-      <c r="D240" s="3"/>
-      <c r="E240" s="3"/>
-      <c r="F240" s="3"/>
-      <c r="G240" s="3"/>
-      <c r="H240" s="3"/>
+      <c r="A240" s="2" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="s">
@@ -3305,8 +4250,8 @@
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="s">
-        <v>161</v>
+      <c r="A242" s="4" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="243">
@@ -3314,15 +4259,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" ht="8" customHeight="true">
-      <c r="A244" s="17"/>
-      <c r="B244" s="17"/>
-      <c r="C244" s="17"/>
-      <c r="D244" s="17"/>
-      <c r="E244" s="17"/>
-      <c r="F244" s="17"/>
-      <c r="G244" s="17"/>
-      <c r="H244" s="17"/>
+    <row r="244">
+      <c r="A244" s="2" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="s">
@@ -3339,15 +4279,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" ht="8" customHeight="true">
-      <c r="A248" s="17"/>
-      <c r="B248" s="17"/>
-      <c r="C248" s="17"/>
-      <c r="D248" s="17"/>
-      <c r="E248" s="17"/>
-      <c r="F248" s="17"/>
-      <c r="G248" s="17"/>
-      <c r="H248" s="17"/>
+    <row r="248">
+      <c r="A248" s="2" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="s">
@@ -3356,7 +4291,7 @@
     </row>
     <row r="250">
       <c r="A250" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="251">
@@ -3364,15 +4299,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" ht="8" customHeight="true">
-      <c r="A252" s="17"/>
-      <c r="B252" s="17"/>
-      <c r="C252" s="17"/>
-      <c r="D252" s="17"/>
-      <c r="E252" s="17"/>
-      <c r="F252" s="17"/>
-      <c r="G252" s="17"/>
-      <c r="H252" s="17"/>
+    <row r="252">
+      <c r="A252" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="s">
@@ -3380,8 +4310,8 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="s">
-        <v>164</v>
+      <c r="A254" s="4" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="255">
@@ -3390,16 +4320,9 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B256" s="3"/>
-      <c r="C256" s="3"/>
-      <c r="D256" s="3"/>
-      <c r="E256" s="3"/>
-      <c r="F256" s="3"/>
-      <c r="G256" s="3"/>
-      <c r="H256" s="3"/>
+      <c r="A256" s="2" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="s">
@@ -3407,8 +4330,8 @@
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="4" t="s">
-        <v>166</v>
+      <c r="A258" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="259">
@@ -3417,28 +4340,28 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="s">
-        <v>167</v>
+      <c r="A260" s="4" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="s">
-        <v>168</v>
+        <v>1</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="s">
-        <v>1</v>
+        <v>171</v>
       </c>
     </row>
     <row r="264">
-      <c r="A264" s="4" t="s">
-        <v>170</v>
+      <c r="A264" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="265">
@@ -3448,7 +4371,7 @@
     </row>
     <row r="266">
       <c r="A266" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="267">
@@ -3458,7 +4381,7 @@
     </row>
     <row r="268">
       <c r="A268" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="269">
@@ -3468,297 +4391,598 @@
     </row>
     <row r="270">
       <c r="A270" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="s">
-        <v>174</v>
+        <v>1</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="s">
-        <v>1</v>
+        <v>176</v>
       </c>
     </row>
     <row r="273">
-      <c r="A273" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B273" s="3"/>
-      <c r="C273" s="3"/>
-      <c r="D273" s="3"/>
-      <c r="E273" s="3"/>
-      <c r="F273" s="3"/>
-      <c r="G273" s="3"/>
-      <c r="H273" s="3"/>
+      <c r="A273" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="s">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="4" t="s">
-        <v>176</v>
+      <c r="A275" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="s">
-        <v>1</v>
+        <v>178</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="s">
-        <v>177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A278" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B278" s="3"/>
+      <c r="C278" s="3"/>
+      <c r="D278" s="3"/>
+      <c r="E278" s="3"/>
+      <c r="F278" s="3"/>
+      <c r="G278" s="3"/>
+      <c r="H278" s="3"/>
     </row>
     <row r="279">
-      <c r="A279" s="4" t="s">
-        <v>178</v>
+      <c r="A279" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="s">
-        <v>1</v>
+        <v>180</v>
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="1" t="s">
-        <v>179</v>
+      <c r="A281" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="s">
-        <v>1</v>
+        <v>181</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="s">
-        <v>180</v>
+        <v>1</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="s">
-        <v>1</v>
+        <v>182</v>
       </c>
     </row>
     <row r="285">
-      <c r="A285" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="B285" s="3"/>
-      <c r="C285" s="3"/>
-      <c r="D285" s="3"/>
-      <c r="E285" s="3"/>
-      <c r="F285" s="3"/>
-      <c r="G285" s="3"/>
-      <c r="H285" s="3"/>
+      <c r="A285" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="s">
-        <v>1</v>
+        <v>183</v>
       </c>
     </row>
     <row r="287">
-      <c r="A287" s="4" t="s">
-        <v>182</v>
+      <c r="A287" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A288" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B288" s="3"/>
+      <c r="C288" s="3"/>
+      <c r="D288" s="3"/>
+      <c r="E288" s="3"/>
+      <c r="F288" s="3"/>
+      <c r="G288" s="3"/>
+      <c r="H288" s="3"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="s">
-        <v>183</v>
+        <v>1</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="s">
-        <v>1</v>
+        <v>185</v>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A291" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292" ht="8" customHeight="true">
+      <c r="A292" s="17"/>
+      <c r="B292" s="17"/>
+      <c r="C292" s="17"/>
+      <c r="D292" s="17"/>
+      <c r="E292" s="17"/>
+      <c r="F292" s="17"/>
+      <c r="G292" s="17"/>
+      <c r="H292" s="17"/>
     </row>
     <row r="293">
       <c r="A293" s="2" t="s">
-        <v>185</v>
+        <v>1</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="s">
-        <v>1</v>
+        <v>186</v>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="6" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A295" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296" ht="8" customHeight="true">
+      <c r="A296" s="17"/>
+      <c r="B296" s="17"/>
+      <c r="C296" s="17"/>
+      <c r="D296" s="17"/>
+      <c r="E296" s="17"/>
+      <c r="F296" s="17"/>
+      <c r="G296" s="17"/>
+      <c r="H296" s="17"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="s">
-        <v>187</v>
+        <v>1</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="s">
-        <v>1</v>
+        <v>187</v>
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="7" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A299" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300" ht="8" customHeight="true">
+      <c r="A300" s="17"/>
+      <c r="B300" s="17"/>
+      <c r="C300" s="17"/>
+      <c r="D300" s="17"/>
+      <c r="E300" s="17"/>
+      <c r="F300" s="17"/>
+      <c r="G300" s="17"/>
+      <c r="H300" s="17"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="s">
-        <v>189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="s">
-        <v>1</v>
+        <v>188</v>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="4" t="s">
-        <v>190</v>
+      <c r="A303" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A304" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B304" s="3"/>
+      <c r="C304" s="3"/>
+      <c r="D304" s="3"/>
+      <c r="E304" s="3"/>
+      <c r="F304" s="3"/>
+      <c r="G304" s="3"/>
+      <c r="H304" s="3"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="s">
-        <v>191</v>
+        <v>1</v>
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="s">
-        <v>1</v>
+      <c r="A306" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B307" s="3"/>
-      <c r="C307" s="3"/>
-      <c r="D307" s="3"/>
-      <c r="E307" s="3"/>
-      <c r="F307" s="3"/>
-      <c r="G307" s="3"/>
-      <c r="H307" s="3"/>
+      <c r="A307" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="s">
-        <v>1</v>
+        <v>191</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="4" t="s">
         <v>194</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="2" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="s">
-        <v>196</v>
+        <v>1</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="s">
-        <v>198</v>
+        <v>1</v>
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="2" t="s">
-        <v>199</v>
+      <c r="A316" s="4" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="s">
-        <v>200</v>
+        <v>1</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="s">
-        <v>203</v>
+        <v>1</v>
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="s">
-        <v>204</v>
-      </c>
+      <c r="A321" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B321" s="3"/>
+      <c r="C321" s="3"/>
+      <c r="D321" s="3"/>
+      <c r="E321" s="3"/>
+      <c r="F321" s="3"/>
+      <c r="G321" s="3"/>
+      <c r="H321" s="3"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="s">
-        <v>205</v>
+        <v>1</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="2" t="s">
-        <v>206</v>
+      <c r="A323" s="4" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B333" s="3"/>
+      <c r="C333" s="3"/>
+      <c r="D333" s="3"/>
+      <c r="E333" s="3"/>
+      <c r="F333" s="3"/>
+      <c r="G333" s="3"/>
+      <c r="H333" s="3"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="5" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B355" s="3"/>
+      <c r="C355" s="3"/>
+      <c r="D355" s="3"/>
+      <c r="E355" s="3"/>
+      <c r="F355" s="3"/>
+      <c r="G355" s="3"/>
+      <c r="H355" s="3"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3776,12 +5000,16 @@
     <mergeCell ref="A118:H120"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A190" r:id="rId1"/>
-    <hyperlink ref="A192" r:id="rId2"/>
-    <hyperlink ref="A194" r:id="rId3"/>
-    <hyperlink ref="A198" r:id="rId4"/>
-    <hyperlink ref="A200" r:id="rId5"/>
-    <hyperlink ref="A202" r:id="rId6"/>
+    <hyperlink ref="A196" r:id="rId1"/>
+    <hyperlink ref="A198" r:id="rId2"/>
+    <hyperlink ref="A200" r:id="rId3"/>
+    <hyperlink ref="A204" r:id="rId4"/>
+    <hyperlink ref="A206" r:id="rId5"/>
+    <hyperlink ref="A208" r:id="rId6"/>
+    <hyperlink ref="A212" r:id="rId7"/>
+    <hyperlink ref="A216" r:id="rId8"/>
+    <hyperlink ref="A218" r:id="rId9"/>
+    <hyperlink ref="A220" r:id="rId10"/>
   </hyperlinks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add init subcommand and change default sheet name
  - Add  to generate .m2x.yml with all config options
    and explanatory comments; skips if file already exists
  - Change default sheet_name from doc to Sheet1
  - Handle Sheet1 rename correctly in renderer when using default name
</commit_message>
<xml_diff>
--- a/sample/output/demo.xlsx
+++ b/sample/output/demo.xlsx
@@ -7,7 +7,7 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="doc" sheetId="2" r:id="rId4"/>
+    <sheet name="Sample" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -2241,7 +2241,7 @@
       <family val="2"/>
       <b val="1"/>
       <color/>
-      <sz val="24"/>
+      <sz val="32"/>
     </font>
     <font>
       <name val="游ゴシック Regular"/>

</xml_diff>

<commit_message>
Fix sample md file
</commit_message>
<xml_diff>
--- a/sample/output/demo.xlsx
+++ b/sample/output/demo.xlsx
@@ -2435,6 +2435,122 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>127</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7010400" cy="7010400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>130</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>132</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7010400" cy="7010400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>135</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>914400</xdr:colOff>
+      <xdr:row>137</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 4" descr=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7010400" cy="7010400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:ln/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="true" fPrintsWithSheet="true"/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3656,500 +3772,484 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
+    <row r="126" ht="409" customHeight="true"/>
+    <row r="127" ht="204.5" customHeight="true"/>
     <row r="128">
-      <c r="A128" s="4" t="s">
+      <c r="A128" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="4" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
+    <row r="130">
+      <c r="A130" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" ht="409" customHeight="true"/>
+    <row r="132" ht="204.5" customHeight="true"/>
     <row r="133">
       <c r="A133" s="2" t="s">
         <v>1</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
     <row r="135">
       <c r="A135" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="3" t="s">
+    <row r="136" ht="409" customHeight="true"/>
+    <row r="137" ht="204.5" customHeight="true"/>
+    <row r="138">
+      <c r="A138" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="3"/>
-      <c r="F136" s="3"/>
-      <c r="G136" s="3"/>
-      <c r="H136" s="3"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="B139" s="3"/>
+      <c r="C139" s="3"/>
+      <c r="D139" s="3"/>
+      <c r="E139" s="3"/>
+      <c r="F139" s="3"/>
+      <c r="G139" s="3"/>
+      <c r="H139" s="3"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="s">
-        <v>94</v>
+        <v>1</v>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="s">
-        <v>95</v>
+      <c r="A141" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="s">
-        <v>96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="s">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="4" t="s">
-        <v>103</v>
+      <c r="A150" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="s">
-        <v>1</v>
+        <v>102</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="s">
-        <v>104</v>
+        <v>1</v>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="s">
-        <v>105</v>
+      <c r="A153" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="s">
-        <v>106</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="s">
-        <v>1</v>
+        <v>104</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="4" t="s">
-        <v>107</v>
+      <c r="A156" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="s">
-        <v>1</v>
+        <v>106</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="s">
-        <v>108</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="s">
-        <v>109</v>
+      <c r="A159" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="s">
-        <v>110</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="s">
-        <v>1</v>
+        <v>113</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="4" t="s">
-        <v>116</v>
+      <c r="A167" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="s">
-        <v>1</v>
+        <v>115</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="s">
-        <v>117</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="s">
-        <v>118</v>
+      <c r="A170" s="4" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="s">
-        <v>119</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="s">
-        <v>1</v>
+        <v>119</v>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="4" t="s">
-        <v>122</v>
+      <c r="A175" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="s">
-        <v>1</v>
+        <v>121</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="s">
-        <v>123</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="s">
-        <v>124</v>
+      <c r="A178" s="4" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="s">
-        <v>125</v>
+        <v>1</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="s">
-        <v>1</v>
+        <v>129</v>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="4" t="s">
-        <v>132</v>
+      <c r="A187" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="s">
-        <v>1</v>
+        <v>131</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="s">
-        <v>133</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="s">
-        <v>134</v>
+      <c r="A190" s="4" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="s">
-        <v>135</v>
+        <v>1</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="s">
-        <v>1</v>
+        <v>134</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B194" s="3"/>
-      <c r="C194" s="3"/>
-      <c r="D194" s="3"/>
-      <c r="E194" s="3"/>
-      <c r="F194" s="3"/>
-      <c r="G194" s="3"/>
-      <c r="H194" s="3"/>
+      <c r="A194" s="2" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="s">
-        <v>1</v>
+        <v>136</v>
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="16" t="s">
+      <c r="A196" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B197" s="3"/>
+      <c r="C197" s="3"/>
+      <c r="D197" s="3"/>
+      <c r="E197" s="3"/>
+      <c r="F197" s="3"/>
+      <c r="G197" s="3"/>
+      <c r="H197" s="3"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="16" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="16" t="s">
+    <row r="200">
+      <c r="A200" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="16" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="16" t="s">
+    <row r="202">
+      <c r="A202" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="16" t="s">
         <v>140</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="4" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="2" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="s">
-        <v>142</v>
+        <v>1</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="s">
-        <v>1</v>
+      <c r="A205" s="4" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="s">
-        <v>143</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="s">
-        <v>1</v>
+        <v>142</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="s">
-        <v>144</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="s">
-        <v>1</v>
+        <v>143</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="4" t="s">
-        <v>145</v>
+      <c r="A210" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="s">
-        <v>1</v>
+        <v>144</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="16" t="s">
+      <c r="A212" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="4" t="s">
+    <row r="216">
+      <c r="A216" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="4" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" s="16" t="s">
+    <row r="218">
+      <c r="A218" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="16" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="16" t="s">
+    <row r="220">
+      <c r="A220" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="16" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" s="16" t="s">
+    <row r="222">
+      <c r="A222" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="16" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B222" s="3"/>
-      <c r="C222" s="3"/>
-      <c r="D222" s="3"/>
-      <c r="E222" s="3"/>
-      <c r="F222" s="3"/>
-      <c r="G222" s="3"/>
-      <c r="H222" s="3"/>
-    </row>
-    <row r="223">
-      <c r="A223" s="2" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="224">
@@ -4158,9 +4258,16 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="s">
-        <v>152</v>
-      </c>
+      <c r="A225" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B225" s="3"/>
+      <c r="C225" s="3"/>
+      <c r="D225" s="3"/>
+      <c r="E225" s="3"/>
+      <c r="F225" s="3"/>
+      <c r="G225" s="3"/>
+      <c r="H225" s="3"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="s">
@@ -4173,16 +4280,9 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B228" s="3"/>
-      <c r="C228" s="3"/>
-      <c r="D228" s="3"/>
-      <c r="E228" s="3"/>
-      <c r="F228" s="3"/>
-      <c r="G228" s="3"/>
-      <c r="H228" s="3"/>
+      <c r="A228" s="2" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="s">
@@ -4191,488 +4291,495 @@
     </row>
     <row r="230">
       <c r="A230" s="2" t="s">
-        <v>154</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A231" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B231" s="3"/>
+      <c r="C231" s="3"/>
+      <c r="D231" s="3"/>
+      <c r="E231" s="3"/>
+      <c r="F231" s="3"/>
+      <c r="G231" s="3"/>
+      <c r="H231" s="3"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="s">
-        <v>155</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="s">
-        <v>1</v>
+        <v>154</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="s">
-        <v>156</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="s">
-        <v>1</v>
+        <v>155</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="s">
-        <v>157</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="s">
-        <v>1</v>
+        <v>156</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="s">
-        <v>158</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="s">
-        <v>1</v>
+        <v>157</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="s">
-        <v>159</v>
+        <v>1</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="s">
-        <v>1</v>
+        <v>158</v>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="4" t="s">
-        <v>160</v>
+      <c r="A242" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="s">
-        <v>1</v>
+        <v>159</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="s">
-        <v>161</v>
+        <v>1</v>
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="s">
-        <v>1</v>
+      <c r="A245" s="4" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="s">
-        <v>162</v>
+        <v>1</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="s">
-        <v>1</v>
+        <v>161</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="s">
-        <v>163</v>
+        <v>1</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="s">
-        <v>1</v>
+        <v>162</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="s">
-        <v>164</v>
+        <v>1</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="s">
-        <v>1</v>
+        <v>163</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="s">
-        <v>165</v>
+        <v>1</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="2" t="s">
-        <v>1</v>
+        <v>164</v>
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="4" t="s">
-        <v>166</v>
+      <c r="A254" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="s">
-        <v>1</v>
+        <v>165</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="2" t="s">
-        <v>167</v>
+        <v>1</v>
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="s">
-        <v>1</v>
+      <c r="A257" s="4" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="2" t="s">
-        <v>168</v>
+        <v>1</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="s">
-        <v>1</v>
+        <v>167</v>
       </c>
     </row>
     <row r="260">
-      <c r="A260" s="4" t="s">
-        <v>169</v>
+      <c r="A260" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="s">
-        <v>1</v>
+        <v>168</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="s">
-        <v>170</v>
+        <v>1</v>
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="s">
-        <v>171</v>
+      <c r="A263" s="4" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="s">
-        <v>172</v>
+        <v>1</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="s">
-        <v>1</v>
+        <v>170</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="s">
-        <v>1</v>
+        <v>172</v>
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="4" t="s">
-        <v>174</v>
+      <c r="A268" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="s">
-        <v>1</v>
+        <v>173</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="s">
-        <v>175</v>
+        <v>1</v>
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="s">
-        <v>1</v>
+      <c r="A271" s="4" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="s">
-        <v>176</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="s">
-        <v>1</v>
+        <v>175</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="s">
-        <v>177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="s">
-        <v>1</v>
+        <v>176</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="s">
-        <v>178</v>
+        <v>1</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="s">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="278">
-      <c r="A278" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="B278" s="3"/>
-      <c r="C278" s="3"/>
-      <c r="D278" s="3"/>
-      <c r="E278" s="3"/>
-      <c r="F278" s="3"/>
-      <c r="G278" s="3"/>
-      <c r="H278" s="3"/>
+      <c r="A278" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="s">
-        <v>1</v>
+        <v>178</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="s">
-        <v>180</v>
+        <v>1</v>
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A281" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B281" s="3"/>
+      <c r="C281" s="3"/>
+      <c r="D281" s="3"/>
+      <c r="E281" s="3"/>
+      <c r="F281" s="3"/>
+      <c r="G281" s="3"/>
+      <c r="H281" s="3"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="s">
-        <v>181</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="2" t="s">
-        <v>1</v>
+        <v>180</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="2" t="s">
-        <v>182</v>
+        <v>1</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="2" t="s">
-        <v>1</v>
+        <v>181</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="s">
-        <v>183</v>
+        <v>1</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="2" t="s">
-        <v>1</v>
+        <v>182</v>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B288" s="3"/>
-      <c r="C288" s="3"/>
-      <c r="D288" s="3"/>
-      <c r="E288" s="3"/>
-      <c r="F288" s="3"/>
-      <c r="G288" s="3"/>
-      <c r="H288" s="3"/>
+      <c r="A288" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="s">
-        <v>1</v>
+        <v>183</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="s">
-        <v>185</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="292" ht="8" customHeight="true">
-      <c r="A292" s="17"/>
-      <c r="B292" s="17"/>
-      <c r="C292" s="17"/>
-      <c r="D292" s="17"/>
-      <c r="E292" s="17"/>
-      <c r="F292" s="17"/>
-      <c r="G292" s="17"/>
-      <c r="H292" s="17"/>
+      <c r="A291" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B291" s="3"/>
+      <c r="C291" s="3"/>
+      <c r="D291" s="3"/>
+      <c r="E291" s="3"/>
+      <c r="F291" s="3"/>
+      <c r="G291" s="3"/>
+      <c r="H291" s="3"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="s">
-        <v>1</v>
+        <v>185</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="296" ht="8" customHeight="true">
-      <c r="A296" s="17"/>
-      <c r="B296" s="17"/>
-      <c r="C296" s="17"/>
-      <c r="D296" s="17"/>
-      <c r="E296" s="17"/>
-      <c r="F296" s="17"/>
-      <c r="G296" s="17"/>
-      <c r="H296" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295" ht="8" customHeight="true">
+      <c r="A295" s="17"/>
+      <c r="B295" s="17"/>
+      <c r="C295" s="17"/>
+      <c r="D295" s="17"/>
+      <c r="E295" s="17"/>
+      <c r="F295" s="17"/>
+      <c r="G295" s="17"/>
+      <c r="H295" s="17"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="s">
-        <v>1</v>
+        <v>186</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="300" ht="8" customHeight="true">
-      <c r="A300" s="17"/>
-      <c r="B300" s="17"/>
-      <c r="C300" s="17"/>
-      <c r="D300" s="17"/>
-      <c r="E300" s="17"/>
-      <c r="F300" s="17"/>
-      <c r="G300" s="17"/>
-      <c r="H300" s="17"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299" ht="8" customHeight="true">
+      <c r="A299" s="17"/>
+      <c r="B299" s="17"/>
+      <c r="C299" s="17"/>
+      <c r="D299" s="17"/>
+      <c r="E299" s="17"/>
+      <c r="F299" s="17"/>
+      <c r="G299" s="17"/>
+      <c r="H299" s="17"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="s">
-        <v>1</v>
+        <v>187</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" s="2" t="s">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303" ht="8" customHeight="true">
+      <c r="A303" s="17"/>
+      <c r="B303" s="17"/>
+      <c r="C303" s="17"/>
+      <c r="D303" s="17"/>
+      <c r="E303" s="17"/>
+      <c r="F303" s="17"/>
+      <c r="G303" s="17"/>
+      <c r="H303" s="17"/>
     </row>
     <row r="304">
-      <c r="A304" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="B304" s="3"/>
-      <c r="C304" s="3"/>
-      <c r="D304" s="3"/>
-      <c r="E304" s="3"/>
-      <c r="F304" s="3"/>
-      <c r="G304" s="3"/>
-      <c r="H304" s="3"/>
+      <c r="A304" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="s">
-        <v>1</v>
+        <v>188</v>
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="4" t="s">
-        <v>190</v>
+      <c r="A306" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A307" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B307" s="3"/>
+      <c r="C307" s="3"/>
+      <c r="D307" s="3"/>
+      <c r="E307" s="3"/>
+      <c r="F307" s="3"/>
+      <c r="G307" s="3"/>
+      <c r="H307" s="3"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="s">
-        <v>191</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="2" t="s">
-        <v>192</v>
+      <c r="A309" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="s">
-        <v>193</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="s">
-        <v>1</v>
+        <v>191</v>
       </c>
     </row>
     <row r="312">
-      <c r="A312" s="4" t="s">
-        <v>194</v>
+      <c r="A312" s="2" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="s">
-        <v>1</v>
+        <v>193</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="s">
-        <v>195</v>
+        <v>1</v>
       </c>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="s">
-        <v>1</v>
+      <c r="A315" s="4" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="316">
-      <c r="A316" s="4" t="s">
-        <v>196</v>
+      <c r="A316" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="s">
-        <v>1</v>
+        <v>195</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="s">
-        <v>197</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="s">
-        <v>198</v>
+      <c r="A319" s="4" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="320">
@@ -4681,308 +4788,323 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B321" s="3"/>
-      <c r="C321" s="3"/>
-      <c r="D321" s="3"/>
-      <c r="E321" s="3"/>
-      <c r="F321" s="3"/>
-      <c r="G321" s="3"/>
-      <c r="H321" s="3"/>
+      <c r="A321" s="2" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="s">
-        <v>1</v>
+        <v>198</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="4" t="s">
-        <v>200</v>
+      <c r="A323" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A324" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B324" s="3"/>
+      <c r="C324" s="3"/>
+      <c r="D324" s="3"/>
+      <c r="E324" s="3"/>
+      <c r="F324" s="3"/>
+      <c r="G324" s="3"/>
+      <c r="H324" s="3"/>
     </row>
     <row r="325">
       <c r="A325" s="2" t="s">
-        <v>201</v>
+        <v>1</v>
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="2" t="s">
-        <v>1</v>
+      <c r="A326" s="4" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="4" t="s">
-        <v>202</v>
+      <c r="A327" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="s">
-        <v>1</v>
+        <v>201</v>
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="1" t="s">
-        <v>203</v>
+      <c r="A329" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="2" t="s">
-        <v>1</v>
+      <c r="A330" s="4" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="s">
-        <v>204</v>
+        <v>1</v>
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="s">
-        <v>1</v>
+      <c r="A332" s="1" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="333">
-      <c r="A333" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B333" s="3"/>
-      <c r="C333" s="3"/>
-      <c r="D333" s="3"/>
-      <c r="E333" s="3"/>
-      <c r="F333" s="3"/>
-      <c r="G333" s="3"/>
-      <c r="H333" s="3"/>
+      <c r="A333" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="s">
-        <v>1</v>
+        <v>204</v>
       </c>
     </row>
     <row r="335">
-      <c r="A335" s="4" t="s">
-        <v>206</v>
+      <c r="A335" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="336">
-      <c r="A336" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A336" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B336" s="3"/>
+      <c r="C336" s="3"/>
+      <c r="D336" s="3"/>
+      <c r="E336" s="3"/>
+      <c r="F336" s="3"/>
+      <c r="G336" s="3"/>
+      <c r="H336" s="3"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="s">
-        <v>207</v>
+        <v>1</v>
       </c>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="s">
-        <v>1</v>
+      <c r="A338" s="4" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="5" t="s">
-        <v>208</v>
+      <c r="A339" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="s">
-        <v>1</v>
+        <v>207</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="s">
-        <v>209</v>
+        <v>1</v>
       </c>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="s">
-        <v>1</v>
+      <c r="A342" s="5" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="6" t="s">
-        <v>210</v>
+      <c r="A343" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="s">
-        <v>1</v>
+        <v>209</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="s">
-        <v>211</v>
+        <v>1</v>
       </c>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="s">
-        <v>1</v>
+      <c r="A346" s="6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="347">
-      <c r="A347" s="7" t="s">
-        <v>212</v>
+      <c r="A347" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="s">
-        <v>1</v>
+        <v>211</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="s">
-        <v>213</v>
+        <v>1</v>
       </c>
     </row>
     <row r="350">
-      <c r="A350" s="2" t="s">
-        <v>1</v>
+      <c r="A350" s="7" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="351">
-      <c r="A351" s="4" t="s">
-        <v>214</v>
+      <c r="A351" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="s">
-        <v>1</v>
+        <v>213</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="s">
-        <v>215</v>
+        <v>1</v>
       </c>
     </row>
     <row r="354">
-      <c r="A354" s="2" t="s">
-        <v>1</v>
+      <c r="A354" s="4" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="355">
-      <c r="A355" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B355" s="3"/>
-      <c r="C355" s="3"/>
-      <c r="D355" s="3"/>
-      <c r="E355" s="3"/>
-      <c r="F355" s="3"/>
-      <c r="G355" s="3"/>
-      <c r="H355" s="3"/>
+      <c r="A355" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="s">
-        <v>1</v>
+        <v>215</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="s">
-        <v>217</v>
+        <v>1</v>
       </c>
     </row>
     <row r="358">
-      <c r="A358" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A358" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B358" s="3"/>
+      <c r="C358" s="3"/>
+      <c r="D358" s="3"/>
+      <c r="E358" s="3"/>
+      <c r="F358" s="3"/>
+      <c r="G358" s="3"/>
+      <c r="H358" s="3"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="s">
-        <v>218</v>
+        <v>1</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="s">
-        <v>220</v>
+        <v>1</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -5000,16 +5122,17 @@
     <mergeCell ref="A118:H120"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A196" r:id="rId1"/>
-    <hyperlink ref="A198" r:id="rId2"/>
-    <hyperlink ref="A200" r:id="rId3"/>
-    <hyperlink ref="A204" r:id="rId4"/>
-    <hyperlink ref="A206" r:id="rId5"/>
-    <hyperlink ref="A208" r:id="rId6"/>
-    <hyperlink ref="A212" r:id="rId7"/>
-    <hyperlink ref="A216" r:id="rId8"/>
-    <hyperlink ref="A218" r:id="rId9"/>
-    <hyperlink ref="A220" r:id="rId10"/>
+    <hyperlink ref="A199" r:id="rId2"/>
+    <hyperlink ref="A201" r:id="rId3"/>
+    <hyperlink ref="A203" r:id="rId4"/>
+    <hyperlink ref="A207" r:id="rId5"/>
+    <hyperlink ref="A209" r:id="rId6"/>
+    <hyperlink ref="A211" r:id="rId7"/>
+    <hyperlink ref="A215" r:id="rId8"/>
+    <hyperlink ref="A219" r:id="rId9"/>
+    <hyperlink ref="A221" r:id="rId10"/>
+    <hyperlink ref="A223" r:id="rId11"/>
   </hyperlinks>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add rich text rendering in table cells
  Preserve bold, italic, strikethrough, and code font formatting
  in table header and data cells instead of stripping to plain text.
  Add demo section with inline formatting examples in tables.
</commit_message>
<xml_diff>
--- a/sample/output/demo.xlsx
+++ b/sample/output/demo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
   <si>
     <t>1. md2xls Feature Demo</t>
   </si>
@@ -372,7 +372,33 @@
     <t>Blockquotes</t>
   </si>
   <si>
-    <t>Consecutive `&gt;` lines grouped</t>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve">Consecutive </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> lines grouped</t>
+    </r>
   </si>
   <si>
     <t>Images</t>
@@ -483,7 +509,176 @@
     <t>C+</t>
   </si>
   <si>
-    <t>1.2.4. Wide Column Table</t>
+    <t>1.2.4. Table with Inline Formatting</t>
+  </si>
+  <si>
+    <t>Syntax</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Bold</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>bold text</t>
+    </r>
+  </si>
+  <si>
+    <t>Markers stripped</t>
+  </si>
+  <si>
+    <t>Italic</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <i val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>italic text</t>
+    </r>
+  </si>
+  <si>
+    <t>Inline code</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>code text</t>
+    </r>
+  </si>
+  <si>
+    <t>Strikethrough</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <strike val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>deleted</t>
+    </r>
+  </si>
+  <si>
+    <t>Underscore bold</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>bold</t>
+    </r>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>example</t>
+  </si>
+  <si>
+    <t>Link text only</t>
+  </si>
+  <si>
+    <t>Mixed</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t>bold</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>code</t>
+    </r>
+  </si>
+  <si>
+    <t>Both stripped</t>
+  </si>
+  <si>
+    <t>HTML entity</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="游ゴシック Regular"/>
+        <family val="2"/>
+        <color/>
+        <sz val="11"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <color/>
+        <sz val="10.5"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+  </si>
+  <si>
+    <t>Decoded</t>
+  </si>
+  <si>
+    <t>1.2.5. Wide Column Table</t>
   </si>
   <si>
     <t>Description</t>
@@ -2443,13 +2638,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>125</xdr:row>
+      <xdr:row>137</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>127</xdr:row>
+      <xdr:row>139</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2480,13 +2675,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>130</xdr:row>
+      <xdr:row>142</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>132</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2517,13 +2712,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>135</xdr:row>
+      <xdr:row>147</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
       <xdr:colOff>914400</xdr:colOff>
-      <xdr:row>137</xdr:row>
+      <xdr:row>149</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -3270,163 +3465,170 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B67" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C67" s="8"/>
-    </row>
-    <row r="68" ht="105" customHeight="true">
-      <c r="A68" s="9" t="s">
+      <c r="B79" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C79" s="8"/>
+    </row>
+    <row r="80" ht="105" customHeight="true">
+      <c r="A80" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B68" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C68" s="9"/>
-    </row>
-    <row r="69" ht="105" customHeight="true">
-      <c r="A69" s="9" t="s">
+      <c r="B80" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C80" s="9"/>
+    </row>
+    <row r="81" ht="105" customHeight="true">
+      <c r="A81" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B69" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C69" s="9"/>
-    </row>
-    <row r="70" ht="105" customHeight="true">
-      <c r="A70" s="9" t="s">
+      <c r="B81" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C81" s="9"/>
+    </row>
+    <row r="82" ht="105" customHeight="true">
+      <c r="A82" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B70" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C70" s="9"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B76" s="14"/>
-      <c r="C76" s="14"/>
-      <c r="D76" s="14"/>
-      <c r="E76" s="14"/>
-      <c r="F76" s="14"/>
-      <c r="G76" s="14"/>
-      <c r="H76" s="14"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="14"/>
-      <c r="B77" s="14"/>
-      <c r="C77" s="14"/>
-      <c r="D77" s="14"/>
-      <c r="E77" s="14"/>
-      <c r="F77" s="14"/>
-      <c r="G77" s="14"/>
-      <c r="H77" s="14"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="14"/>
-      <c r="B78" s="14"/>
-      <c r="C78" s="14"/>
-      <c r="D78" s="14"/>
-      <c r="E78" s="14"/>
-      <c r="F78" s="14"/>
-      <c r="G78" s="14"/>
-      <c r="H78" s="14"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="14"/>
-      <c r="B79" s="14"/>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
-      <c r="F79" s="14"/>
-      <c r="G79" s="14"/>
-      <c r="H79" s="14"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="14"/>
-      <c r="B80" s="14"/>
-      <c r="C80" s="14"/>
-      <c r="D80" s="14"/>
-      <c r="E80" s="14"/>
-      <c r="F80" s="14"/>
-      <c r="G80" s="14"/>
-      <c r="H80" s="14"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="14"/>
-      <c r="B81" s="14"/>
-      <c r="C81" s="14"/>
-      <c r="D81" s="14"/>
-      <c r="E81" s="14"/>
-      <c r="F81" s="14"/>
-      <c r="G81" s="14"/>
-      <c r="H81" s="14"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="14"/>
-      <c r="B82" s="14"/>
-      <c r="C82" s="14"/>
-      <c r="D82" s="14"/>
-      <c r="E82" s="14"/>
-      <c r="F82" s="14"/>
-      <c r="G82" s="14"/>
-      <c r="H82" s="14"/>
+      <c r="B82" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C82" s="9"/>
     </row>
     <row r="83">
-      <c r="A83" s="14"/>
-      <c r="B83" s="14"/>
-      <c r="C83" s="14"/>
-      <c r="D83" s="14"/>
-      <c r="E83" s="14"/>
-      <c r="F83" s="14"/>
-      <c r="G83" s="14"/>
-      <c r="H83" s="14"/>
+      <c r="A83" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="14"/>
-      <c r="B84" s="14"/>
-      <c r="C84" s="14"/>
-      <c r="D84" s="14"/>
-      <c r="E84" s="14"/>
-      <c r="F84" s="14"/>
-      <c r="G84" s="14"/>
-      <c r="H84" s="14"/>
+      <c r="A84" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="H84" s="3"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="s">
@@ -3435,7 +3637,7 @@
     </row>
     <row r="86">
       <c r="A86" s="4" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
     </row>
     <row r="87">
@@ -3445,7 +3647,7 @@
     </row>
     <row r="88">
       <c r="A88" s="14" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="B88" s="14"/>
       <c r="C88" s="14"/>
@@ -3526,34 +3728,34 @@
       <c r="H95" s="14"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A96" s="14"/>
+      <c r="B96" s="14"/>
+      <c r="C96" s="14"/>
+      <c r="D96" s="14"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="14"/>
+      <c r="G96" s="14"/>
+      <c r="H96" s="14"/>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="s">
-        <v>81</v>
+      <c r="A97" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="s">
-        <v>1</v>
+      <c r="A98" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="B99" s="14"/>
-      <c r="C99" s="14"/>
-      <c r="D99" s="14"/>
-      <c r="E99" s="14"/>
-      <c r="F99" s="14"/>
-      <c r="G99" s="14"/>
-      <c r="H99" s="14"/>
+      <c r="A99" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="14"/>
+      <c r="A100" s="14" t="s">
+        <v>104</v>
+      </c>
       <c r="B100" s="14"/>
       <c r="C100" s="14"/>
       <c r="D100" s="14"/>
@@ -3583,125 +3785,128 @@
       <c r="H102" s="14"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A103" s="14"/>
+      <c r="B103" s="14"/>
+      <c r="C103" s="14"/>
+      <c r="D103" s="14"/>
+      <c r="E103" s="14"/>
+      <c r="F103" s="14"/>
+      <c r="G103" s="14"/>
+      <c r="H103" s="14"/>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
-      <c r="G104" s="3"/>
-      <c r="H104" s="3"/>
+      <c r="A104" s="14"/>
+      <c r="B104" s="14"/>
+      <c r="C104" s="14"/>
+      <c r="D104" s="14"/>
+      <c r="E104" s="14"/>
+      <c r="F104" s="14"/>
+      <c r="G104" s="14"/>
+      <c r="H104" s="14"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A105" s="14"/>
+      <c r="B105" s="14"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="14"/>
+      <c r="E105" s="14"/>
+      <c r="F105" s="14"/>
+      <c r="G105" s="14"/>
+      <c r="H105" s="14"/>
     </row>
     <row r="106">
-      <c r="A106" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B106" s="15"/>
-      <c r="C106" s="15"/>
-      <c r="D106" s="15"/>
-      <c r="E106" s="15"/>
-      <c r="F106" s="15"/>
-      <c r="G106" s="15"/>
-      <c r="H106" s="15"/>
+      <c r="A106" s="14"/>
+      <c r="B106" s="14"/>
+      <c r="C106" s="14"/>
+      <c r="D106" s="14"/>
+      <c r="E106" s="14"/>
+      <c r="F106" s="14"/>
+      <c r="G106" s="14"/>
+      <c r="H106" s="14"/>
     </row>
     <row r="107">
-      <c r="A107" s="15"/>
-      <c r="B107" s="15"/>
-      <c r="C107" s="15"/>
-      <c r="D107" s="15"/>
-      <c r="E107" s="15"/>
-      <c r="F107" s="15"/>
-      <c r="G107" s="15"/>
-      <c r="H107" s="15"/>
+      <c r="A107" s="14"/>
+      <c r="B107" s="14"/>
+      <c r="C107" s="14"/>
+      <c r="D107" s="14"/>
+      <c r="E107" s="14"/>
+      <c r="F107" s="14"/>
+      <c r="G107" s="14"/>
+      <c r="H107" s="14"/>
     </row>
     <row r="108">
-      <c r="A108" s="15"/>
-      <c r="B108" s="15"/>
-      <c r="C108" s="15"/>
-      <c r="D108" s="15"/>
-      <c r="E108" s="15"/>
-      <c r="F108" s="15"/>
-      <c r="G108" s="15"/>
-      <c r="H108" s="15"/>
+      <c r="A108" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="15"/>
-      <c r="B109" s="15"/>
-      <c r="C109" s="15"/>
-      <c r="D109" s="15"/>
-      <c r="E109" s="15"/>
-      <c r="F109" s="15"/>
-      <c r="G109" s="15"/>
-      <c r="H109" s="15"/>
+      <c r="A109" s="4" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="15"/>
-      <c r="B110" s="15"/>
-      <c r="C110" s="15"/>
-      <c r="D110" s="15"/>
-      <c r="E110" s="15"/>
-      <c r="F110" s="15"/>
-      <c r="G110" s="15"/>
-      <c r="H110" s="15"/>
+      <c r="A110" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A111" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B111" s="14"/>
+      <c r="C111" s="14"/>
+      <c r="D111" s="14"/>
+      <c r="E111" s="14"/>
+      <c r="F111" s="14"/>
+      <c r="G111" s="14"/>
+      <c r="H111" s="14"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="s">
-        <v>85</v>
-      </c>
+      <c r="A112" s="14"/>
+      <c r="B112" s="14"/>
+      <c r="C112" s="14"/>
+      <c r="D112" s="14"/>
+      <c r="E112" s="14"/>
+      <c r="F112" s="14"/>
+      <c r="G112" s="14"/>
+      <c r="H112" s="14"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A113" s="14"/>
+      <c r="B113" s="14"/>
+      <c r="C113" s="14"/>
+      <c r="D113" s="14"/>
+      <c r="E113" s="14"/>
+      <c r="F113" s="14"/>
+      <c r="G113" s="14"/>
+      <c r="H113" s="14"/>
     </row>
     <row r="114">
-      <c r="A114" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="B114" s="15"/>
-      <c r="C114" s="15"/>
-      <c r="D114" s="15"/>
-      <c r="E114" s="15"/>
-      <c r="F114" s="15"/>
-      <c r="G114" s="15"/>
-      <c r="H114" s="15"/>
+      <c r="A114" s="14"/>
+      <c r="B114" s="14"/>
+      <c r="C114" s="14"/>
+      <c r="D114" s="14"/>
+      <c r="E114" s="14"/>
+      <c r="F114" s="14"/>
+      <c r="G114" s="14"/>
+      <c r="H114" s="14"/>
     </row>
     <row r="115">
-      <c r="A115" s="15"/>
-      <c r="B115" s="15"/>
-      <c r="C115" s="15"/>
-      <c r="D115" s="15"/>
-      <c r="E115" s="15"/>
-      <c r="F115" s="15"/>
-      <c r="G115" s="15"/>
-      <c r="H115" s="15"/>
+      <c r="A115" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="15"/>
-      <c r="B116" s="15"/>
-      <c r="C116" s="15"/>
-      <c r="D116" s="15"/>
-      <c r="E116" s="15"/>
-      <c r="F116" s="15"/>
-      <c r="G116" s="15"/>
-      <c r="H116" s="15"/>
+      <c r="A116" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B116" s="3"/>
+      <c r="C116" s="3"/>
+      <c r="D116" s="3"/>
+      <c r="E116" s="3"/>
+      <c r="F116" s="3"/>
+      <c r="G116" s="3"/>
+      <c r="H116" s="3"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="s">
@@ -3710,7 +3915,7 @@
     </row>
     <row r="118">
       <c r="A118" s="15" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -3741,21 +3946,24 @@
       <c r="H120" s="15"/>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A121" s="15"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="15"/>
+      <c r="G121" s="15"/>
+      <c r="H121" s="15"/>
     </row>
     <row r="122">
-      <c r="A122" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B122" s="3"/>
-      <c r="C122" s="3"/>
-      <c r="D122" s="3"/>
-      <c r="E122" s="3"/>
-      <c r="F122" s="3"/>
-      <c r="G122" s="3"/>
-      <c r="H122" s="3"/>
+      <c r="A122" s="15"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="15"/>
+      <c r="F122" s="15"/>
+      <c r="G122" s="15"/>
+      <c r="H122" s="15"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="s">
@@ -3763,8 +3971,8 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="s">
-        <v>89</v>
+      <c r="A124" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="125">
@@ -3772,59 +3980,109 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" ht="409" customHeight="true"/>
-    <row r="127" ht="204.5" customHeight="true"/>
+    <row r="126">
+      <c r="A126" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="15"/>
+      <c r="E126" s="15"/>
+      <c r="F126" s="15"/>
+      <c r="G126" s="15"/>
+      <c r="H126" s="15"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="15"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="15"/>
+      <c r="E127" s="15"/>
+      <c r="F127" s="15"/>
+      <c r="G127" s="15"/>
+      <c r="H127" s="15"/>
+    </row>
     <row r="128">
-      <c r="A128" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A128" s="15"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="15"/>
+      <c r="E128" s="15"/>
+      <c r="F128" s="15"/>
+      <c r="G128" s="15"/>
+      <c r="H128" s="15"/>
     </row>
     <row r="129">
-      <c r="A129" s="4" t="s">
-        <v>90</v>
+      <c r="A129" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="131" ht="409" customHeight="true"/>
-    <row r="132" ht="204.5" customHeight="true"/>
+      <c r="A130" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="B130" s="15"/>
+      <c r="C130" s="15"/>
+      <c r="D130" s="15"/>
+      <c r="E130" s="15"/>
+      <c r="F130" s="15"/>
+      <c r="G130" s="15"/>
+      <c r="H130" s="15"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="15"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="15"/>
+      <c r="E131" s="15"/>
+      <c r="F131" s="15"/>
+      <c r="G131" s="15"/>
+      <c r="H131" s="15"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="15"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="15"/>
+      <c r="E132" s="15"/>
+      <c r="F132" s="15"/>
+      <c r="G132" s="15"/>
+      <c r="H132" s="15"/>
+    </row>
     <row r="133">
       <c r="A133" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="4" t="s">
-        <v>91</v>
-      </c>
+      <c r="A134" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B134" s="3"/>
+      <c r="C134" s="3"/>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3"/>
+      <c r="G134" s="3"/>
+      <c r="H134" s="3"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="136" ht="409" customHeight="true"/>
-    <row r="137" ht="204.5" customHeight="true"/>
-    <row r="138">
-      <c r="A138" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B139" s="3"/>
-      <c r="C139" s="3"/>
-      <c r="D139" s="3"/>
-      <c r="E139" s="3"/>
-      <c r="F139" s="3"/>
-      <c r="G139" s="3"/>
-      <c r="H139" s="3"/>
-    </row>
+    <row r="136">
+      <c r="A136" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" ht="409" customHeight="true"/>
+    <row r="139" ht="204.5" customHeight="true"/>
     <row r="140">
       <c r="A140" s="2" t="s">
         <v>1</v>
@@ -3832,7 +4090,7 @@
     </row>
     <row r="141">
       <c r="A141" s="4" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
     </row>
     <row r="142">
@@ -3840,50 +4098,41 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
+    <row r="143" ht="409" customHeight="true"/>
+    <row r="144" ht="204.5" customHeight="true"/>
     <row r="145">
       <c r="A145" s="2" t="s">
-        <v>96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="s">
-        <v>97</v>
+      <c r="A146" s="4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" ht="409" customHeight="true"/>
+    <row r="149" ht="204.5" customHeight="true"/>
     <row r="150">
       <c r="A150" s="2" t="s">
-        <v>101</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="s">
-        <v>102</v>
-      </c>
+      <c r="A151" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B151" s="3"/>
+      <c r="C151" s="3"/>
+      <c r="D151" s="3"/>
+      <c r="E151" s="3"/>
+      <c r="F151" s="3"/>
+      <c r="G151" s="3"/>
+      <c r="H151" s="3"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="s">
@@ -3892,7 +4141,7 @@
     </row>
     <row r="153">
       <c r="A153" s="4" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
     </row>
     <row r="154">
@@ -3902,172 +4151,172 @@
     </row>
     <row r="155">
       <c r="A155" s="2" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="s">
-        <v>1</v>
+        <v>121</v>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="4" t="s">
-        <v>107</v>
+      <c r="A159" s="2" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="s">
-        <v>1</v>
+        <v>123</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="s">
-        <v>111</v>
+        <v>1</v>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="s">
-        <v>112</v>
+      <c r="A165" s="4" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="s">
-        <v>113</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="s">
-        <v>1</v>
+        <v>130</v>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="4" t="s">
-        <v>116</v>
+      <c r="A170" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="s">
-        <v>1</v>
+      <c r="A171" s="4" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="s">
-        <v>117</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="s">
-        <v>1</v>
+        <v>136</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="4" t="s">
-        <v>122</v>
+      <c r="A178" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="s">
-        <v>1</v>
+        <v>138</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="s">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="s">
-        <v>125</v>
+      <c r="A182" s="4" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="s">
-        <v>126</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
     </row>
     <row r="189">
@@ -4077,7 +4326,7 @@
     </row>
     <row r="190">
       <c r="A190" s="4" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
     </row>
     <row r="191">
@@ -4087,89 +4336,82 @@
     </row>
     <row r="192">
       <c r="A192" s="2" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B197" s="3"/>
-      <c r="C197" s="3"/>
-      <c r="D197" s="3"/>
-      <c r="E197" s="3"/>
-      <c r="F197" s="3"/>
-      <c r="G197" s="3"/>
-      <c r="H197" s="3"/>
+      <c r="A197" s="2" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="s">
-        <v>1</v>
+        <v>153</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="16" t="s">
-        <v>138</v>
+      <c r="A199" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="s">
-        <v>1</v>
+        <v>155</v>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="16" t="s">
-        <v>139</v>
+      <c r="A201" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="s">
-        <v>1</v>
+      <c r="A202" s="4" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="16" t="s">
-        <v>140</v>
+      <c r="A203" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="s">
-        <v>1</v>
+        <v>157</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="4" t="s">
-        <v>141</v>
+      <c r="A205" s="2" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="s">
-        <v>1</v>
+        <v>159</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
     </row>
     <row r="208">
@@ -4178,9 +4420,16 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="s">
-        <v>143</v>
-      </c>
+      <c r="A209" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B209" s="3"/>
+      <c r="C209" s="3"/>
+      <c r="D209" s="3"/>
+      <c r="E209" s="3"/>
+      <c r="F209" s="3"/>
+      <c r="G209" s="3"/>
+      <c r="H209" s="3"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="s">
@@ -4188,8 +4437,8 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="s">
-        <v>144</v>
+      <c r="A211" s="16" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="212">
@@ -4198,8 +4447,8 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="4" t="s">
-        <v>145</v>
+      <c r="A213" s="16" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="214">
@@ -4209,7 +4458,7 @@
     </row>
     <row r="215">
       <c r="A215" s="16" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
     </row>
     <row r="216">
@@ -4219,7 +4468,7 @@
     </row>
     <row r="217">
       <c r="A217" s="4" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
     </row>
     <row r="218">
@@ -4228,8 +4477,8 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="16" t="s">
-        <v>148</v>
+      <c r="A219" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="220">
@@ -4238,8 +4487,8 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="16" t="s">
-        <v>149</v>
+      <c r="A221" s="2" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="222">
@@ -4248,8 +4497,8 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="16" t="s">
-        <v>150</v>
+      <c r="A223" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="224">
@@ -4258,16 +4507,9 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="B225" s="3"/>
-      <c r="C225" s="3"/>
-      <c r="D225" s="3"/>
-      <c r="E225" s="3"/>
-      <c r="F225" s="3"/>
-      <c r="G225" s="3"/>
-      <c r="H225" s="3"/>
+      <c r="A225" s="4" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="s">
@@ -4275,18 +4517,18 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="s">
-        <v>1</v>
+      <c r="A227" s="16" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="s">
-        <v>152</v>
+        <v>1</v>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="s">
-        <v>1</v>
+      <c r="A229" s="4" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="230">
@@ -4295,16 +4537,9 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B231" s="3"/>
-      <c r="C231" s="3"/>
-      <c r="D231" s="3"/>
-      <c r="E231" s="3"/>
-      <c r="F231" s="3"/>
-      <c r="G231" s="3"/>
-      <c r="H231" s="3"/>
+      <c r="A231" s="16" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="s">
@@ -4312,8 +4547,8 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="s">
-        <v>154</v>
+      <c r="A233" s="16" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="234">
@@ -4322,8 +4557,8 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="s">
-        <v>155</v>
+      <c r="A235" s="16" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="236">
@@ -4332,9 +4567,16 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="s">
-        <v>156</v>
-      </c>
+      <c r="A237" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B237" s="3"/>
+      <c r="C237" s="3"/>
+      <c r="D237" s="3"/>
+      <c r="E237" s="3"/>
+      <c r="F237" s="3"/>
+      <c r="G237" s="3"/>
+      <c r="H237" s="3"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="s">
@@ -4343,17 +4585,17 @@
     </row>
     <row r="239">
       <c r="A239" s="2" t="s">
-        <v>157</v>
+        <v>1</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="s">
-        <v>1</v>
+        <v>176</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="s">
-        <v>158</v>
+        <v>1</v>
       </c>
     </row>
     <row r="242">
@@ -4362,9 +4604,16 @@
       </c>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="s">
-        <v>159</v>
-      </c>
+      <c r="A243" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B243" s="3"/>
+      <c r="C243" s="3"/>
+      <c r="D243" s="3"/>
+      <c r="E243" s="3"/>
+      <c r="F243" s="3"/>
+      <c r="G243" s="3"/>
+      <c r="H243" s="3"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="s">
@@ -4372,8 +4621,8 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="4" t="s">
-        <v>160</v>
+      <c r="A245" s="2" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="246">
@@ -4383,7 +4632,7 @@
     </row>
     <row r="247">
       <c r="A247" s="2" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
     </row>
     <row r="248">
@@ -4393,7 +4642,7 @@
     </row>
     <row r="249">
       <c r="A249" s="2" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="250">
@@ -4403,7 +4652,7 @@
     </row>
     <row r="251">
       <c r="A251" s="2" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
     </row>
     <row r="252">
@@ -4413,7 +4662,7 @@
     </row>
     <row r="253">
       <c r="A253" s="2" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
     </row>
     <row r="254">
@@ -4423,7 +4672,7 @@
     </row>
     <row r="255">
       <c r="A255" s="2" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
     </row>
     <row r="256">
@@ -4433,7 +4682,7 @@
     </row>
     <row r="257">
       <c r="A257" s="4" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
     </row>
     <row r="258">
@@ -4443,7 +4692,7 @@
     </row>
     <row r="259">
       <c r="A259" s="2" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
     </row>
     <row r="260">
@@ -4453,7 +4702,7 @@
     </row>
     <row r="261">
       <c r="A261" s="2" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
     </row>
     <row r="262">
@@ -4462,8 +4711,8 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="4" t="s">
-        <v>169</v>
+      <c r="A263" s="2" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="264">
@@ -4473,17 +4722,17 @@
     </row>
     <row r="265">
       <c r="A265" s="2" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="s">
-        <v>171</v>
+        <v>1</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="2" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
     </row>
     <row r="268">
@@ -4492,8 +4741,8 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="s">
-        <v>173</v>
+      <c r="A269" s="4" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="270">
@@ -4502,8 +4751,8 @@
       </c>
     </row>
     <row r="271">
-      <c r="A271" s="4" t="s">
-        <v>174</v>
+      <c r="A271" s="2" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="272">
@@ -4513,7 +4762,7 @@
     </row>
     <row r="273">
       <c r="A273" s="2" t="s">
-        <v>175</v>
+        <v>192</v>
       </c>
     </row>
     <row r="274">
@@ -4522,8 +4771,8 @@
       </c>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="s">
-        <v>176</v>
+      <c r="A275" s="4" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="276">
@@ -4533,17 +4782,17 @@
     </row>
     <row r="277">
       <c r="A277" s="2" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="s">
-        <v>1</v>
+        <v>195</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
     </row>
     <row r="280">
@@ -4552,16 +4801,9 @@
       </c>
     </row>
     <row r="281">
-      <c r="A281" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="B281" s="3"/>
-      <c r="C281" s="3"/>
-      <c r="D281" s="3"/>
-      <c r="E281" s="3"/>
-      <c r="F281" s="3"/>
-      <c r="G281" s="3"/>
-      <c r="H281" s="3"/>
+      <c r="A281" s="2" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="s">
@@ -4569,8 +4811,8 @@
       </c>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="s">
-        <v>180</v>
+      <c r="A283" s="4" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="284">
@@ -4580,7 +4822,7 @@
     </row>
     <row r="285">
       <c r="A285" s="2" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
     </row>
     <row r="286">
@@ -4590,7 +4832,7 @@
     </row>
     <row r="287">
       <c r="A287" s="2" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
     </row>
     <row r="288">
@@ -4600,7 +4842,7 @@
     </row>
     <row r="289">
       <c r="A289" s="2" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
     </row>
     <row r="290">
@@ -4609,16 +4851,9 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B291" s="3"/>
-      <c r="C291" s="3"/>
-      <c r="D291" s="3"/>
-      <c r="E291" s="3"/>
-      <c r="F291" s="3"/>
-      <c r="G291" s="3"/>
-      <c r="H291" s="3"/>
+      <c r="A291" s="2" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="s">
@@ -4626,24 +4861,26 @@
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="s">
-        <v>185</v>
-      </c>
+      <c r="A293" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B293" s="3"/>
+      <c r="C293" s="3"/>
+      <c r="D293" s="3"/>
+      <c r="E293" s="3"/>
+      <c r="F293" s="3"/>
+      <c r="G293" s="3"/>
+      <c r="H293" s="3"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="295" ht="8" customHeight="true">
-      <c r="A295" s="17"/>
-      <c r="B295" s="17"/>
-      <c r="C295" s="17"/>
-      <c r="D295" s="17"/>
-      <c r="E295" s="17"/>
-      <c r="F295" s="17"/>
-      <c r="G295" s="17"/>
-      <c r="H295" s="17"/>
+    <row r="295">
+      <c r="A295" s="2" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="2" t="s">
@@ -4652,7 +4889,7 @@
     </row>
     <row r="297">
       <c r="A297" s="2" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
     </row>
     <row r="298">
@@ -4660,15 +4897,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" ht="8" customHeight="true">
-      <c r="A299" s="17"/>
-      <c r="B299" s="17"/>
-      <c r="C299" s="17"/>
-      <c r="D299" s="17"/>
-      <c r="E299" s="17"/>
-      <c r="F299" s="17"/>
-      <c r="G299" s="17"/>
-      <c r="H299" s="17"/>
+    <row r="299">
+      <c r="A299" s="2" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="s">
@@ -4677,7 +4909,7 @@
     </row>
     <row r="301">
       <c r="A301" s="2" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
     </row>
     <row r="302">
@@ -4685,15 +4917,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" ht="8" customHeight="true">
-      <c r="A303" s="17"/>
-      <c r="B303" s="17"/>
-      <c r="C303" s="17"/>
-      <c r="D303" s="17"/>
-      <c r="E303" s="17"/>
-      <c r="F303" s="17"/>
-      <c r="G303" s="17"/>
-      <c r="H303" s="17"/>
+    <row r="303">
+      <c r="A303" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B303" s="3"/>
+      <c r="C303" s="3"/>
+      <c r="D303" s="3"/>
+      <c r="E303" s="3"/>
+      <c r="F303" s="3"/>
+      <c r="G303" s="3"/>
+      <c r="H303" s="3"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="s">
@@ -4702,7 +4936,7 @@
     </row>
     <row r="305">
       <c r="A305" s="2" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
     </row>
     <row r="306">
@@ -4710,17 +4944,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307">
-      <c r="A307" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="B307" s="3"/>
-      <c r="C307" s="3"/>
-      <c r="D307" s="3"/>
-      <c r="E307" s="3"/>
-      <c r="F307" s="3"/>
-      <c r="G307" s="3"/>
-      <c r="H307" s="3"/>
+    <row r="307" ht="8" customHeight="true">
+      <c r="A307" s="17"/>
+      <c r="B307" s="17"/>
+      <c r="C307" s="17"/>
+      <c r="D307" s="17"/>
+      <c r="E307" s="17"/>
+      <c r="F307" s="17"/>
+      <c r="G307" s="17"/>
+      <c r="H307" s="17"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="s">
@@ -4728,8 +4960,8 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="4" t="s">
-        <v>190</v>
+      <c r="A309" s="2" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="310">
@@ -4737,19 +4969,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="311">
-      <c r="A311" s="2" t="s">
-        <v>191</v>
-      </c>
+    <row r="311" ht="8" customHeight="true">
+      <c r="A311" s="17"/>
+      <c r="B311" s="17"/>
+      <c r="C311" s="17"/>
+      <c r="D311" s="17"/>
+      <c r="E311" s="17"/>
+      <c r="F311" s="17"/>
+      <c r="G311" s="17"/>
+      <c r="H311" s="17"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="s">
-        <v>192</v>
+        <v>1</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
     </row>
     <row r="314">
@@ -4757,10 +4994,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315">
-      <c r="A315" s="4" t="s">
-        <v>194</v>
-      </c>
+    <row r="315" ht="8" customHeight="true">
+      <c r="A315" s="17"/>
+      <c r="B315" s="17"/>
+      <c r="C315" s="17"/>
+      <c r="D315" s="17"/>
+      <c r="E315" s="17"/>
+      <c r="F315" s="17"/>
+      <c r="G315" s="17"/>
+      <c r="H315" s="17"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="s">
@@ -4769,7 +5011,7 @@
     </row>
     <row r="317">
       <c r="A317" s="2" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
     </row>
     <row r="318">
@@ -4778,9 +5020,16 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="4" t="s">
-        <v>196</v>
-      </c>
+      <c r="A319" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B319" s="3"/>
+      <c r="C319" s="3"/>
+      <c r="D319" s="3"/>
+      <c r="E319" s="3"/>
+      <c r="F319" s="3"/>
+      <c r="G319" s="3"/>
+      <c r="H319" s="3"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="s">
@@ -4788,80 +5037,73 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="s">
-        <v>197</v>
+      <c r="A321" s="4" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="s">
-        <v>198</v>
+        <v>1</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="s">
-        <v>1</v>
+        <v>215</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B324" s="3"/>
-      <c r="C324" s="3"/>
-      <c r="D324" s="3"/>
-      <c r="E324" s="3"/>
-      <c r="F324" s="3"/>
-      <c r="G324" s="3"/>
-      <c r="H324" s="3"/>
+      <c r="A324" s="2" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="s">
-        <v>1</v>
+        <v>217</v>
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="4" t="s">
-        <v>200</v>
+      <c r="A326" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="327">
-      <c r="A327" s="2" t="s">
-        <v>1</v>
+      <c r="A327" s="4" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="s">
-        <v>201</v>
+        <v>1</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="s">
-        <v>1</v>
+        <v>219</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" s="4" t="s">
-        <v>202</v>
+      <c r="A330" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="s">
-        <v>1</v>
+      <c r="A331" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="332">
-      <c r="A332" s="1" t="s">
-        <v>203</v>
+      <c r="A332" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="s">
-        <v>1</v>
+        <v>221</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
     </row>
     <row r="335">
@@ -4871,7 +5113,7 @@
     </row>
     <row r="336">
       <c r="A336" s="3" t="s">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="B336" s="3"/>
       <c r="C336" s="3"/>
@@ -4888,7 +5130,7 @@
     </row>
     <row r="338">
       <c r="A338" s="4" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
     </row>
     <row r="339">
@@ -4898,7 +5140,7 @@
     </row>
     <row r="340">
       <c r="A340" s="2" t="s">
-        <v>207</v>
+        <v>225</v>
       </c>
     </row>
     <row r="341">
@@ -4907,8 +5149,8 @@
       </c>
     </row>
     <row r="342">
-      <c r="A342" s="5" t="s">
-        <v>208</v>
+      <c r="A342" s="4" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="343">
@@ -4917,8 +5159,8 @@
       </c>
     </row>
     <row r="344">
-      <c r="A344" s="2" t="s">
-        <v>209</v>
+      <c r="A344" s="1" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="345">
@@ -4927,8 +5169,8 @@
       </c>
     </row>
     <row r="346">
-      <c r="A346" s="6" t="s">
-        <v>210</v>
+      <c r="A346" s="2" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="347">
@@ -4937,9 +5179,16 @@
       </c>
     </row>
     <row r="348">
-      <c r="A348" s="2" t="s">
-        <v>211</v>
-      </c>
+      <c r="A348" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B348" s="3"/>
+      <c r="C348" s="3"/>
+      <c r="D348" s="3"/>
+      <c r="E348" s="3"/>
+      <c r="F348" s="3"/>
+      <c r="G348" s="3"/>
+      <c r="H348" s="3"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="s">
@@ -4947,8 +5196,8 @@
       </c>
     </row>
     <row r="350">
-      <c r="A350" s="7" t="s">
-        <v>212</v>
+      <c r="A350" s="4" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="351">
@@ -4958,7 +5207,7 @@
     </row>
     <row r="352">
       <c r="A352" s="2" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
     </row>
     <row r="353">
@@ -4967,8 +5216,8 @@
       </c>
     </row>
     <row r="354">
-      <c r="A354" s="4" t="s">
-        <v>214</v>
+      <c r="A354" s="5" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="355">
@@ -4978,7 +5227,7 @@
     </row>
     <row r="356">
       <c r="A356" s="2" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
     </row>
     <row r="357">
@@ -4987,16 +5236,9 @@
       </c>
     </row>
     <row r="358">
-      <c r="A358" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B358" s="3"/>
-      <c r="C358" s="3"/>
-      <c r="D358" s="3"/>
-      <c r="E358" s="3"/>
-      <c r="F358" s="3"/>
-      <c r="G358" s="3"/>
-      <c r="H358" s="3"/>
+      <c r="A358" s="6" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="s">
@@ -5005,7 +5247,7 @@
     </row>
     <row r="360">
       <c r="A360" s="2" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
     </row>
     <row r="361">
@@ -5014,124 +5256,191 @@
       </c>
     </row>
     <row r="362">
-      <c r="A362" s="2" t="s">
-        <v>218</v>
+      <c r="A362" s="7" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="s">
-        <v>219</v>
+        <v>1</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="2" t="s">
-        <v>221</v>
+        <v>1</v>
       </c>
     </row>
     <row r="366">
-      <c r="A366" s="2" t="s">
-        <v>222</v>
+      <c r="A366" s="4" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="s">
-        <v>223</v>
+        <v>1</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="s">
-        <v>225</v>
+        <v>1</v>
       </c>
     </row>
     <row r="370">
-      <c r="A370" s="2" t="s">
-        <v>226</v>
-      </c>
+      <c r="A370" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B370" s="3"/>
+      <c r="C370" s="3"/>
+      <c r="D370" s="3"/>
+      <c r="E370" s="3"/>
+      <c r="F370" s="3"/>
+      <c r="G370" s="3"/>
+      <c r="H370" s="3"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="s">
-        <v>227</v>
+        <v>1</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="s">
-        <v>229</v>
+        <v>1</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="A76:H84"/>
-    <mergeCell ref="A88:H95"/>
-    <mergeCell ref="A99:H102"/>
-    <mergeCell ref="A106:H110"/>
-    <mergeCell ref="A114:H116"/>
-    <mergeCell ref="A118:H120"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="A88:H96"/>
+    <mergeCell ref="A100:H107"/>
+    <mergeCell ref="A111:H114"/>
+    <mergeCell ref="A118:H122"/>
+    <mergeCell ref="A126:H128"/>
+    <mergeCell ref="A130:H132"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A199" r:id="rId2"/>
-    <hyperlink ref="A201" r:id="rId3"/>
-    <hyperlink ref="A203" r:id="rId4"/>
-    <hyperlink ref="A207" r:id="rId5"/>
-    <hyperlink ref="A209" r:id="rId6"/>
-    <hyperlink ref="A211" r:id="rId7"/>
-    <hyperlink ref="A215" r:id="rId8"/>
-    <hyperlink ref="A219" r:id="rId9"/>
-    <hyperlink ref="A221" r:id="rId10"/>
-    <hyperlink ref="A223" r:id="rId11"/>
+    <hyperlink ref="A211" r:id="rId2"/>
+    <hyperlink ref="A213" r:id="rId3"/>
+    <hyperlink ref="A215" r:id="rId4"/>
+    <hyperlink ref="A219" r:id="rId5"/>
+    <hyperlink ref="A221" r:id="rId6"/>
+    <hyperlink ref="A223" r:id="rId7"/>
+    <hyperlink ref="A227" r:id="rId8"/>
+    <hyperlink ref="A231" r:id="rId9"/>
+    <hyperlink ref="A233" r:id="rId10"/>
+    <hyperlink ref="A235" r:id="rId11"/>
   </hyperlinks>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>